<commit_message>
Update logic slice layout
</commit_message>
<xml_diff>
--- a/Configuration Generator/Layout Drawings.xlsx
+++ b/Configuration Generator/Layout Drawings.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/13561f3231cadc0a/DTU/Comp_Arch_2/eFPGA/Configuration Generator/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="778" documentId="13_ncr:1_{FB05B031-63D2-4F22-8938-A1D344FEFB29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E9F0A7C2-AE61-43F7-AEE6-C38EA2A38A27}"/>
+  <xr:revisionPtr revIDLastSave="799" documentId="13_ncr:1_{FB05B031-63D2-4F22-8938-A1D344FEFB29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E5385872-9F90-499E-BA0B-8143A08ADF97}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Logic_Slice" sheetId="4" r:id="rId1"/>
@@ -356,10 +356,10 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
+      <left style="medium">
         <color indexed="64"/>
       </left>
-      <right style="medium">
+      <right style="thin">
         <color indexed="64"/>
       </right>
       <top style="thin">
@@ -398,10 +398,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1399,10 +1399,10 @@
       <c r="B7" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C7" t="s">
-        <v>6</v>
-      </c>
-      <c r="D7" t="s">
+      <c r="C7" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="D7" s="25" t="s">
         <v>6</v>
       </c>
       <c r="E7" s="5" t="s">
@@ -1468,10 +1468,10 @@
       <c r="AA7" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="AB7" t="s">
-        <v>6</v>
-      </c>
-      <c r="AC7" t="s">
+      <c r="AB7" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="AC7" s="25" t="s">
         <v>6</v>
       </c>
       <c r="AD7" s="5" t="s">
@@ -1537,10 +1537,10 @@
       <c r="AZ7" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="BA7" t="s">
-        <v>6</v>
-      </c>
-      <c r="BB7" t="s">
+      <c r="BA7" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="BB7" s="25" t="s">
         <v>6</v>
       </c>
       <c r="BC7" s="5" t="s">
@@ -1606,10 +1606,10 @@
       <c r="BY7" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="BZ7" t="s">
-        <v>6</v>
-      </c>
-      <c r="CA7" t="s">
+      <c r="BZ7" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="CA7" s="25" t="s">
         <v>6</v>
       </c>
       <c r="CB7" s="5" t="s">
@@ -1623,10 +1623,10 @@
       <c r="B8" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C8" t="s">
-        <v>6</v>
-      </c>
-      <c r="D8" t="s">
+      <c r="C8" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="D8" s="25" t="s">
         <v>6</v>
       </c>
       <c r="E8" s="5" t="s">
@@ -1692,10 +1692,10 @@
       <c r="AA8" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="AB8" t="s">
-        <v>6</v>
-      </c>
-      <c r="AC8" t="s">
+      <c r="AB8" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="AC8" s="25" t="s">
         <v>6</v>
       </c>
       <c r="AD8" s="5" t="s">
@@ -1761,10 +1761,10 @@
       <c r="AZ8" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="BA8" t="s">
-        <v>6</v>
-      </c>
-      <c r="BB8" t="s">
+      <c r="BA8" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="BB8" s="25" t="s">
         <v>6</v>
       </c>
       <c r="BC8" s="5" t="s">
@@ -1830,10 +1830,10 @@
       <c r="BY8" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="BZ8" t="s">
-        <v>6</v>
-      </c>
-      <c r="CA8" t="s">
+      <c r="BZ8" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="CA8" s="25" t="s">
         <v>6</v>
       </c>
       <c r="CB8" s="5" t="s">
@@ -1847,10 +1847,10 @@
       <c r="B9" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C9" t="s">
-        <v>6</v>
-      </c>
-      <c r="D9" t="s">
+      <c r="C9" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="D9" s="25" t="s">
         <v>6</v>
       </c>
       <c r="E9" s="5" t="s">
@@ -1916,10 +1916,10 @@
       <c r="AA9" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="AB9" t="s">
-        <v>6</v>
-      </c>
-      <c r="AC9" t="s">
+      <c r="AB9" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="AC9" s="25" t="s">
         <v>6</v>
       </c>
       <c r="AD9" s="5" t="s">
@@ -1985,10 +1985,10 @@
       <c r="AZ9" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="BA9" t="s">
-        <v>6</v>
-      </c>
-      <c r="BB9" t="s">
+      <c r="BA9" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="BB9" s="25" t="s">
         <v>6</v>
       </c>
       <c r="BC9" s="5" t="s">
@@ -2054,10 +2054,10 @@
       <c r="BY9" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="BZ9" t="s">
-        <v>6</v>
-      </c>
-      <c r="CA9" t="s">
+      <c r="BZ9" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="CA9" s="25" t="s">
         <v>6</v>
       </c>
       <c r="CB9" s="5" t="s">
@@ -2071,10 +2071,10 @@
       <c r="B10" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C10" t="s">
-        <v>6</v>
-      </c>
-      <c r="D10" t="s">
+      <c r="C10" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="D10" s="25" t="s">
         <v>6</v>
       </c>
       <c r="E10" s="5" t="s">
@@ -2140,10 +2140,10 @@
       <c r="AA10" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="AB10" t="s">
-        <v>6</v>
-      </c>
-      <c r="AC10" t="s">
+      <c r="AB10" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="AC10" s="25" t="s">
         <v>6</v>
       </c>
       <c r="AD10" s="5" t="s">
@@ -2209,10 +2209,10 @@
       <c r="AZ10" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="BA10" t="s">
-        <v>6</v>
-      </c>
-      <c r="BB10" t="s">
+      <c r="BA10" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="BB10" s="25" t="s">
         <v>6</v>
       </c>
       <c r="BC10" s="5" t="s">
@@ -2278,10 +2278,10 @@
       <c r="BY10" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="BZ10" t="s">
-        <v>6</v>
-      </c>
-      <c r="CA10" t="s">
+      <c r="BZ10" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="CA10" s="25" t="s">
         <v>6</v>
       </c>
       <c r="CB10" s="5" t="s">
@@ -2295,10 +2295,10 @@
       <c r="B11" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C11" t="s">
-        <v>6</v>
-      </c>
-      <c r="D11" t="s">
+      <c r="C11" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="D11" s="25" t="s">
         <v>6</v>
       </c>
       <c r="E11" s="5" t="s">
@@ -2364,10 +2364,10 @@
       <c r="AA11" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="AB11" t="s">
-        <v>6</v>
-      </c>
-      <c r="AC11" t="s">
+      <c r="AB11" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="AC11" s="25" t="s">
         <v>6</v>
       </c>
       <c r="AD11" s="5" t="s">
@@ -2433,10 +2433,10 @@
       <c r="AZ11" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="BA11" t="s">
-        <v>6</v>
-      </c>
-      <c r="BB11" t="s">
+      <c r="BA11" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="BB11" s="25" t="s">
         <v>6</v>
       </c>
       <c r="BC11" s="5" t="s">
@@ -2502,10 +2502,10 @@
       <c r="BY11" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="BZ11" t="s">
-        <v>6</v>
-      </c>
-      <c r="CA11" t="s">
+      <c r="BZ11" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="CA11" s="25" t="s">
         <v>6</v>
       </c>
       <c r="CB11" s="5" t="s">
@@ -2516,10 +2516,10 @@
       <c r="B12" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C12" t="s">
-        <v>6</v>
-      </c>
-      <c r="D12" t="s">
+      <c r="C12" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="D12" s="25" t="s">
         <v>6</v>
       </c>
       <c r="E12" s="5" t="s">
@@ -2558,10 +2558,10 @@
       <c r="AA12" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="AB12" t="s">
-        <v>6</v>
-      </c>
-      <c r="AC12" t="s">
+      <c r="AB12" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="AC12" s="25" t="s">
         <v>6</v>
       </c>
       <c r="AD12" s="5" t="s">
@@ -2600,10 +2600,10 @@
       <c r="AZ12" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="BA12" t="s">
-        <v>6</v>
-      </c>
-      <c r="BB12" t="s">
+      <c r="BA12" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="BB12" s="25" t="s">
         <v>6</v>
       </c>
       <c r="BC12" s="5" t="s">
@@ -2642,10 +2642,10 @@
       <c r="BY12" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="BZ12" t="s">
-        <v>6</v>
-      </c>
-      <c r="CA12" t="s">
+      <c r="BZ12" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="CA12" s="25" t="s">
         <v>6</v>
       </c>
       <c r="CB12" s="5" t="s">
@@ -2820,14 +2820,14 @@
       </c>
     </row>
     <row r="14" spans="1:81" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B14" s="6"/>
-      <c r="C14" s="7"/>
-      <c r="D14" s="22" t="s">
+      <c r="B14" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="E14" s="23" t="s">
+      <c r="C14" s="22" t="s">
         <v>9</v>
       </c>
+      <c r="D14" s="7"/>
+      <c r="E14" s="8"/>
       <c r="F14" t="s">
         <v>8</v>
       </c>
@@ -2867,14 +2867,14 @@
       <c r="Z14" t="s">
         <v>8</v>
       </c>
-      <c r="AA14" s="6"/>
-      <c r="AB14" s="7"/>
-      <c r="AC14" s="22" t="s">
+      <c r="AA14" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="AD14" s="23" t="s">
+      <c r="AB14" s="22" t="s">
         <v>9</v>
       </c>
+      <c r="AC14" s="7"/>
+      <c r="AD14" s="8"/>
       <c r="AE14" t="s">
         <v>8</v>
       </c>
@@ -2914,14 +2914,14 @@
       <c r="AY14" t="s">
         <v>8</v>
       </c>
-      <c r="AZ14" s="6"/>
-      <c r="BA14" s="7"/>
-      <c r="BB14" s="22" t="s">
+      <c r="AZ14" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="BC14" s="23" t="s">
+      <c r="BA14" s="22" t="s">
         <v>9</v>
       </c>
+      <c r="BB14" s="7"/>
+      <c r="BC14" s="8"/>
       <c r="BD14" t="s">
         <v>8</v>
       </c>
@@ -2961,14 +2961,14 @@
       <c r="BX14" t="s">
         <v>8</v>
       </c>
-      <c r="BY14" s="6"/>
-      <c r="BZ14" s="7"/>
-      <c r="CA14" s="22" t="s">
+      <c r="BY14" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="CB14" s="23" t="s">
+      <c r="BZ14" s="22" t="s">
         <v>9</v>
       </c>
+      <c r="CA14" s="7"/>
+      <c r="CB14" s="8"/>
     </row>
     <row r="15" spans="1:81" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A15" s="15"/>
@@ -3534,10 +3534,10 @@
       <c r="B20" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C20" t="s">
-        <v>6</v>
-      </c>
-      <c r="D20" t="s">
+      <c r="C20" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="D20" s="25" t="s">
         <v>6</v>
       </c>
       <c r="E20" s="5" t="s">
@@ -3603,10 +3603,10 @@
       <c r="AA20" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="AB20" t="s">
-        <v>6</v>
-      </c>
-      <c r="AC20" t="s">
+      <c r="AB20" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="AC20" s="25" t="s">
         <v>6</v>
       </c>
       <c r="AD20" s="5" t="s">
@@ -3672,10 +3672,10 @@
       <c r="AZ20" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="BA20" t="s">
-        <v>6</v>
-      </c>
-      <c r="BB20" t="s">
+      <c r="BA20" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="BB20" s="25" t="s">
         <v>6</v>
       </c>
       <c r="BC20" s="5" t="s">
@@ -3741,10 +3741,10 @@
       <c r="BY20" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="BZ20" t="s">
-        <v>6</v>
-      </c>
-      <c r="CA20" t="s">
+      <c r="BZ20" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="CA20" s="25" t="s">
         <v>6</v>
       </c>
       <c r="CB20" s="5" t="s">
@@ -3758,10 +3758,10 @@
       <c r="B21" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C21" t="s">
-        <v>6</v>
-      </c>
-      <c r="D21" t="s">
+      <c r="C21" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="D21" s="25" t="s">
         <v>6</v>
       </c>
       <c r="E21" s="5" t="s">
@@ -3827,10 +3827,10 @@
       <c r="AA21" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="AB21" t="s">
-        <v>6</v>
-      </c>
-      <c r="AC21" t="s">
+      <c r="AB21" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="AC21" s="25" t="s">
         <v>6</v>
       </c>
       <c r="AD21" s="5" t="s">
@@ -3896,10 +3896,10 @@
       <c r="AZ21" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="BA21" t="s">
-        <v>6</v>
-      </c>
-      <c r="BB21" t="s">
+      <c r="BA21" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="BB21" s="25" t="s">
         <v>6</v>
       </c>
       <c r="BC21" s="5" t="s">
@@ -3965,10 +3965,10 @@
       <c r="BY21" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="BZ21" t="s">
-        <v>6</v>
-      </c>
-      <c r="CA21" t="s">
+      <c r="BZ21" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="CA21" s="25" t="s">
         <v>6</v>
       </c>
       <c r="CB21" s="5" t="s">
@@ -3982,10 +3982,10 @@
       <c r="B22" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C22" t="s">
-        <v>6</v>
-      </c>
-      <c r="D22" t="s">
+      <c r="C22" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="D22" s="25" t="s">
         <v>6</v>
       </c>
       <c r="E22" s="5" t="s">
@@ -4051,10 +4051,10 @@
       <c r="AA22" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="AB22" t="s">
-        <v>6</v>
-      </c>
-      <c r="AC22" t="s">
+      <c r="AB22" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="AC22" s="25" t="s">
         <v>6</v>
       </c>
       <c r="AD22" s="5" t="s">
@@ -4120,10 +4120,10 @@
       <c r="AZ22" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="BA22" t="s">
-        <v>6</v>
-      </c>
-      <c r="BB22" t="s">
+      <c r="BA22" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="BB22" s="25" t="s">
         <v>6</v>
       </c>
       <c r="BC22" s="5" t="s">
@@ -4189,10 +4189,10 @@
       <c r="BY22" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="BZ22" t="s">
-        <v>6</v>
-      </c>
-      <c r="CA22" t="s">
+      <c r="BZ22" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="CA22" s="25" t="s">
         <v>6</v>
       </c>
       <c r="CB22" s="5" t="s">
@@ -4206,10 +4206,10 @@
       <c r="B23" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C23" t="s">
-        <v>6</v>
-      </c>
-      <c r="D23" t="s">
+      <c r="C23" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="D23" s="25" t="s">
         <v>6</v>
       </c>
       <c r="E23" s="5" t="s">
@@ -4275,10 +4275,10 @@
       <c r="AA23" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="AB23" t="s">
-        <v>6</v>
-      </c>
-      <c r="AC23" t="s">
+      <c r="AB23" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="AC23" s="25" t="s">
         <v>6</v>
       </c>
       <c r="AD23" s="5" t="s">
@@ -4344,10 +4344,10 @@
       <c r="AZ23" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="BA23" t="s">
-        <v>6</v>
-      </c>
-      <c r="BB23" t="s">
+      <c r="BA23" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="BB23" s="25" t="s">
         <v>6</v>
       </c>
       <c r="BC23" s="5" t="s">
@@ -4413,10 +4413,10 @@
       <c r="BY23" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="BZ23" t="s">
-        <v>6</v>
-      </c>
-      <c r="CA23" t="s">
+      <c r="BZ23" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="CA23" s="25" t="s">
         <v>6</v>
       </c>
       <c r="CB23" s="5" t="s">
@@ -4430,10 +4430,10 @@
       <c r="B24" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C24" t="s">
-        <v>6</v>
-      </c>
-      <c r="D24" t="s">
+      <c r="C24" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="D24" s="25" t="s">
         <v>6</v>
       </c>
       <c r="E24" s="5" t="s">
@@ -4499,10 +4499,10 @@
       <c r="AA24" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="AB24" t="s">
-        <v>6</v>
-      </c>
-      <c r="AC24" t="s">
+      <c r="AB24" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="AC24" s="25" t="s">
         <v>6</v>
       </c>
       <c r="AD24" s="5" t="s">
@@ -4568,10 +4568,10 @@
       <c r="AZ24" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="BA24" t="s">
-        <v>6</v>
-      </c>
-      <c r="BB24" t="s">
+      <c r="BA24" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="BB24" s="25" t="s">
         <v>6</v>
       </c>
       <c r="BC24" s="5" t="s">
@@ -4637,10 +4637,10 @@
       <c r="BY24" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="BZ24" t="s">
-        <v>6</v>
-      </c>
-      <c r="CA24" t="s">
+      <c r="BZ24" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="CA24" s="25" t="s">
         <v>6</v>
       </c>
       <c r="CB24" s="5" t="s">
@@ -4651,10 +4651,10 @@
       <c r="B25" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C25" t="s">
-        <v>6</v>
-      </c>
-      <c r="D25" t="s">
+      <c r="C25" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="D25" s="25" t="s">
         <v>6</v>
       </c>
       <c r="E25" s="5" t="s">
@@ -4693,10 +4693,10 @@
       <c r="AA25" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="AB25" t="s">
-        <v>6</v>
-      </c>
-      <c r="AC25" t="s">
+      <c r="AB25" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="AC25" s="25" t="s">
         <v>6</v>
       </c>
       <c r="AD25" s="5" t="s">
@@ -4735,10 +4735,10 @@
       <c r="AZ25" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="BA25" t="s">
-        <v>6</v>
-      </c>
-      <c r="BB25" t="s">
+      <c r="BA25" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="BB25" s="25" t="s">
         <v>6</v>
       </c>
       <c r="BC25" s="5" t="s">
@@ -4777,10 +4777,10 @@
       <c r="BY25" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="BZ25" t="s">
-        <v>6</v>
-      </c>
-      <c r="CA25" t="s">
+      <c r="BZ25" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="CA25" s="25" t="s">
         <v>6</v>
       </c>
       <c r="CB25" s="5" t="s">
@@ -4955,14 +4955,14 @@
       </c>
     </row>
     <row r="27" spans="1:81" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B27" s="6"/>
-      <c r="C27" s="7"/>
-      <c r="D27" s="22" t="s">
+      <c r="B27" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="E27" s="23" t="s">
+      <c r="C27" s="22" t="s">
         <v>9</v>
       </c>
+      <c r="D27" s="7"/>
+      <c r="E27" s="8"/>
       <c r="F27" t="s">
         <v>8</v>
       </c>
@@ -5002,14 +5002,14 @@
       <c r="Z27" t="s">
         <v>8</v>
       </c>
-      <c r="AA27" s="6"/>
-      <c r="AB27" s="7"/>
-      <c r="AC27" s="22" t="s">
+      <c r="AA27" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="AD27" s="23" t="s">
+      <c r="AB27" s="22" t="s">
         <v>9</v>
       </c>
+      <c r="AC27" s="7"/>
+      <c r="AD27" s="8"/>
       <c r="AE27" t="s">
         <v>8</v>
       </c>
@@ -5049,14 +5049,14 @@
       <c r="AY27" t="s">
         <v>8</v>
       </c>
-      <c r="AZ27" s="6"/>
-      <c r="BA27" s="7"/>
-      <c r="BB27" s="22" t="s">
+      <c r="AZ27" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="BC27" s="23" t="s">
+      <c r="BA27" s="22" t="s">
         <v>9</v>
       </c>
+      <c r="BB27" s="7"/>
+      <c r="BC27" s="8"/>
       <c r="BD27" t="s">
         <v>8</v>
       </c>
@@ -5096,14 +5096,14 @@
       <c r="BX27" t="s">
         <v>8</v>
       </c>
-      <c r="BY27" s="6"/>
-      <c r="BZ27" s="7"/>
-      <c r="CA27" s="22" t="s">
+      <c r="BY27" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="CB27" s="23" t="s">
+      <c r="BZ27" s="22" t="s">
         <v>9</v>
       </c>
+      <c r="CA27" s="7"/>
+      <c r="CB27" s="8"/>
     </row>
     <row r="28" spans="1:81" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A28" s="15"/>
@@ -5669,10 +5669,10 @@
       <c r="B33" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C33" t="s">
-        <v>6</v>
-      </c>
-      <c r="D33" t="s">
+      <c r="C33" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="D33" s="25" t="s">
         <v>6</v>
       </c>
       <c r="E33" s="5" t="s">
@@ -5738,10 +5738,10 @@
       <c r="AA33" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="AB33" t="s">
-        <v>6</v>
-      </c>
-      <c r="AC33" t="s">
+      <c r="AB33" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="AC33" s="25" t="s">
         <v>6</v>
       </c>
       <c r="AD33" s="5" t="s">
@@ -5807,10 +5807,10 @@
       <c r="AZ33" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="BA33" t="s">
-        <v>6</v>
-      </c>
-      <c r="BB33" t="s">
+      <c r="BA33" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="BB33" s="25" t="s">
         <v>6</v>
       </c>
       <c r="BC33" s="5" t="s">
@@ -5876,10 +5876,10 @@
       <c r="BY33" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="BZ33" t="s">
-        <v>6</v>
-      </c>
-      <c r="CA33" t="s">
+      <c r="BZ33" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="CA33" s="25" t="s">
         <v>6</v>
       </c>
       <c r="CB33" s="5" t="s">
@@ -5893,10 +5893,10 @@
       <c r="B34" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C34" t="s">
-        <v>6</v>
-      </c>
-      <c r="D34" t="s">
+      <c r="C34" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="D34" s="25" t="s">
         <v>6</v>
       </c>
       <c r="E34" s="5" t="s">
@@ -5962,10 +5962,10 @@
       <c r="AA34" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="AB34" t="s">
-        <v>6</v>
-      </c>
-      <c r="AC34" t="s">
+      <c r="AB34" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="AC34" s="25" t="s">
         <v>6</v>
       </c>
       <c r="AD34" s="5" t="s">
@@ -6031,10 +6031,10 @@
       <c r="AZ34" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="BA34" t="s">
-        <v>6</v>
-      </c>
-      <c r="BB34" t="s">
+      <c r="BA34" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="BB34" s="25" t="s">
         <v>6</v>
       </c>
       <c r="BC34" s="5" t="s">
@@ -6100,10 +6100,10 @@
       <c r="BY34" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="BZ34" t="s">
-        <v>6</v>
-      </c>
-      <c r="CA34" t="s">
+      <c r="BZ34" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="CA34" s="25" t="s">
         <v>6</v>
       </c>
       <c r="CB34" s="5" t="s">
@@ -6117,10 +6117,10 @@
       <c r="B35" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C35" t="s">
-        <v>6</v>
-      </c>
-      <c r="D35" t="s">
+      <c r="C35" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="D35" s="25" t="s">
         <v>6</v>
       </c>
       <c r="E35" s="5" t="s">
@@ -6186,10 +6186,10 @@
       <c r="AA35" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="AB35" t="s">
-        <v>6</v>
-      </c>
-      <c r="AC35" t="s">
+      <c r="AB35" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="AC35" s="25" t="s">
         <v>6</v>
       </c>
       <c r="AD35" s="5" t="s">
@@ -6255,10 +6255,10 @@
       <c r="AZ35" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="BA35" t="s">
-        <v>6</v>
-      </c>
-      <c r="BB35" t="s">
+      <c r="BA35" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="BB35" s="25" t="s">
         <v>6</v>
       </c>
       <c r="BC35" s="5" t="s">
@@ -6324,10 +6324,10 @@
       <c r="BY35" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="BZ35" t="s">
-        <v>6</v>
-      </c>
-      <c r="CA35" t="s">
+      <c r="BZ35" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="CA35" s="25" t="s">
         <v>6</v>
       </c>
       <c r="CB35" s="5" t="s">
@@ -6341,10 +6341,10 @@
       <c r="B36" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C36" t="s">
-        <v>6</v>
-      </c>
-      <c r="D36" t="s">
+      <c r="C36" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="D36" s="25" t="s">
         <v>6</v>
       </c>
       <c r="E36" s="5" t="s">
@@ -6410,10 +6410,10 @@
       <c r="AA36" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="AB36" t="s">
-        <v>6</v>
-      </c>
-      <c r="AC36" t="s">
+      <c r="AB36" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="AC36" s="25" t="s">
         <v>6</v>
       </c>
       <c r="AD36" s="5" t="s">
@@ -6479,10 +6479,10 @@
       <c r="AZ36" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="BA36" t="s">
-        <v>6</v>
-      </c>
-      <c r="BB36" t="s">
+      <c r="BA36" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="BB36" s="25" t="s">
         <v>6</v>
       </c>
       <c r="BC36" s="5" t="s">
@@ -6548,10 +6548,10 @@
       <c r="BY36" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="BZ36" t="s">
-        <v>6</v>
-      </c>
-      <c r="CA36" t="s">
+      <c r="BZ36" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="CA36" s="25" t="s">
         <v>6</v>
       </c>
       <c r="CB36" s="5" t="s">
@@ -6565,10 +6565,10 @@
       <c r="B37" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C37" t="s">
-        <v>6</v>
-      </c>
-      <c r="D37" t="s">
+      <c r="C37" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="D37" s="25" t="s">
         <v>6</v>
       </c>
       <c r="E37" s="5" t="s">
@@ -6634,10 +6634,10 @@
       <c r="AA37" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="AB37" t="s">
-        <v>6</v>
-      </c>
-      <c r="AC37" t="s">
+      <c r="AB37" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="AC37" s="25" t="s">
         <v>6</v>
       </c>
       <c r="AD37" s="5" t="s">
@@ -6703,10 +6703,10 @@
       <c r="AZ37" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="BA37" t="s">
-        <v>6</v>
-      </c>
-      <c r="BB37" t="s">
+      <c r="BA37" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="BB37" s="25" t="s">
         <v>6</v>
       </c>
       <c r="BC37" s="5" t="s">
@@ -6772,10 +6772,10 @@
       <c r="BY37" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="BZ37" t="s">
-        <v>6</v>
-      </c>
-      <c r="CA37" t="s">
+      <c r="BZ37" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="CA37" s="25" t="s">
         <v>6</v>
       </c>
       <c r="CB37" s="5" t="s">
@@ -6786,10 +6786,10 @@
       <c r="B38" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C38" t="s">
-        <v>6</v>
-      </c>
-      <c r="D38" t="s">
+      <c r="C38" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="D38" s="25" t="s">
         <v>6</v>
       </c>
       <c r="E38" s="5" t="s">
@@ -6828,10 +6828,10 @@
       <c r="AA38" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="AB38" t="s">
-        <v>6</v>
-      </c>
-      <c r="AC38" t="s">
+      <c r="AB38" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="AC38" s="25" t="s">
         <v>6</v>
       </c>
       <c r="AD38" s="5" t="s">
@@ -6870,10 +6870,10 @@
       <c r="AZ38" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="BA38" t="s">
-        <v>6</v>
-      </c>
-      <c r="BB38" t="s">
+      <c r="BA38" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="BB38" s="25" t="s">
         <v>6</v>
       </c>
       <c r="BC38" s="5" t="s">
@@ -6912,10 +6912,10 @@
       <c r="BY38" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="BZ38" t="s">
-        <v>6</v>
-      </c>
-      <c r="CA38" t="s">
+      <c r="BZ38" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="CA38" s="25" t="s">
         <v>6</v>
       </c>
       <c r="CB38" s="5" t="s">
@@ -7090,14 +7090,14 @@
       </c>
     </row>
     <row r="40" spans="1:81" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B40" s="6"/>
-      <c r="C40" s="7"/>
-      <c r="D40" s="22" t="s">
+      <c r="B40" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="E40" s="23" t="s">
+      <c r="C40" s="22" t="s">
         <v>9</v>
       </c>
+      <c r="D40" s="7"/>
+      <c r="E40" s="8"/>
       <c r="F40" t="s">
         <v>8</v>
       </c>
@@ -7137,14 +7137,14 @@
       <c r="Z40" t="s">
         <v>8</v>
       </c>
-      <c r="AA40" s="6"/>
-      <c r="AB40" s="7"/>
-      <c r="AC40" s="22" t="s">
+      <c r="AA40" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="AD40" s="23" t="s">
+      <c r="AB40" s="22" t="s">
         <v>9</v>
       </c>
+      <c r="AC40" s="7"/>
+      <c r="AD40" s="8"/>
       <c r="AE40" t="s">
         <v>8</v>
       </c>
@@ -7184,14 +7184,14 @@
       <c r="AY40" t="s">
         <v>8</v>
       </c>
-      <c r="AZ40" s="6"/>
-      <c r="BA40" s="7"/>
-      <c r="BB40" s="22" t="s">
+      <c r="AZ40" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="BC40" s="23" t="s">
+      <c r="BA40" s="22" t="s">
         <v>9</v>
       </c>
+      <c r="BB40" s="7"/>
+      <c r="BC40" s="8"/>
       <c r="BD40" t="s">
         <v>8</v>
       </c>
@@ -7231,14 +7231,14 @@
       <c r="BX40" t="s">
         <v>8</v>
       </c>
-      <c r="BY40" s="6"/>
-      <c r="BZ40" s="7"/>
-      <c r="CA40" s="22" t="s">
+      <c r="BY40" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="CB40" s="23" t="s">
+      <c r="BZ40" s="22" t="s">
         <v>9</v>
       </c>
+      <c r="CA40" s="7"/>
+      <c r="CB40" s="8"/>
     </row>
     <row r="41" spans="1:81" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A41" s="15"/>
@@ -7804,10 +7804,10 @@
       <c r="B46" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C46" t="s">
-        <v>6</v>
-      </c>
-      <c r="D46" t="s">
+      <c r="C46" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="D46" s="25" t="s">
         <v>6</v>
       </c>
       <c r="E46" s="5" t="s">
@@ -7873,10 +7873,10 @@
       <c r="AA46" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="AB46" t="s">
-        <v>6</v>
-      </c>
-      <c r="AC46" t="s">
+      <c r="AB46" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="AC46" s="25" t="s">
         <v>6</v>
       </c>
       <c r="AD46" s="5" t="s">
@@ -7942,10 +7942,10 @@
       <c r="AZ46" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="BA46" t="s">
-        <v>6</v>
-      </c>
-      <c r="BB46" t="s">
+      <c r="BA46" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="BB46" s="25" t="s">
         <v>6</v>
       </c>
       <c r="BC46" s="5" t="s">
@@ -8011,10 +8011,10 @@
       <c r="BY46" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="BZ46" t="s">
-        <v>6</v>
-      </c>
-      <c r="CA46" t="s">
+      <c r="BZ46" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="CA46" s="25" t="s">
         <v>6</v>
       </c>
       <c r="CB46" s="5" t="s">
@@ -8028,10 +8028,10 @@
       <c r="B47" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C47" t="s">
-        <v>6</v>
-      </c>
-      <c r="D47" t="s">
+      <c r="C47" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="D47" s="25" t="s">
         <v>6</v>
       </c>
       <c r="E47" s="5" t="s">
@@ -8097,10 +8097,10 @@
       <c r="AA47" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="AB47" t="s">
-        <v>6</v>
-      </c>
-      <c r="AC47" t="s">
+      <c r="AB47" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="AC47" s="25" t="s">
         <v>6</v>
       </c>
       <c r="AD47" s="5" t="s">
@@ -8166,10 +8166,10 @@
       <c r="AZ47" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="BA47" t="s">
-        <v>6</v>
-      </c>
-      <c r="BB47" t="s">
+      <c r="BA47" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="BB47" s="25" t="s">
         <v>6</v>
       </c>
       <c r="BC47" s="5" t="s">
@@ -8235,10 +8235,10 @@
       <c r="BY47" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="BZ47" t="s">
-        <v>6</v>
-      </c>
-      <c r="CA47" t="s">
+      <c r="BZ47" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="CA47" s="25" t="s">
         <v>6</v>
       </c>
       <c r="CB47" s="5" t="s">
@@ -8252,10 +8252,10 @@
       <c r="B48" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C48" t="s">
-        <v>6</v>
-      </c>
-      <c r="D48" t="s">
+      <c r="C48" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="D48" s="25" t="s">
         <v>6</v>
       </c>
       <c r="E48" s="5" t="s">
@@ -8321,10 +8321,10 @@
       <c r="AA48" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="AB48" t="s">
-        <v>6</v>
-      </c>
-      <c r="AC48" t="s">
+      <c r="AB48" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="AC48" s="25" t="s">
         <v>6</v>
       </c>
       <c r="AD48" s="5" t="s">
@@ -8390,10 +8390,10 @@
       <c r="AZ48" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="BA48" t="s">
-        <v>6</v>
-      </c>
-      <c r="BB48" t="s">
+      <c r="BA48" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="BB48" s="25" t="s">
         <v>6</v>
       </c>
       <c r="BC48" s="5" t="s">
@@ -8459,10 +8459,10 @@
       <c r="BY48" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="BZ48" t="s">
-        <v>6</v>
-      </c>
-      <c r="CA48" t="s">
+      <c r="BZ48" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="CA48" s="25" t="s">
         <v>6</v>
       </c>
       <c r="CB48" s="5" t="s">
@@ -8476,10 +8476,10 @@
       <c r="B49" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C49" t="s">
-        <v>6</v>
-      </c>
-      <c r="D49" t="s">
+      <c r="C49" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="D49" s="25" t="s">
         <v>6</v>
       </c>
       <c r="E49" s="5" t="s">
@@ -8545,10 +8545,10 @@
       <c r="AA49" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="AB49" t="s">
-        <v>6</v>
-      </c>
-      <c r="AC49" t="s">
+      <c r="AB49" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="AC49" s="25" t="s">
         <v>6</v>
       </c>
       <c r="AD49" s="5" t="s">
@@ -8614,10 +8614,10 @@
       <c r="AZ49" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="BA49" t="s">
-        <v>6</v>
-      </c>
-      <c r="BB49" t="s">
+      <c r="BA49" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="BB49" s="25" t="s">
         <v>6</v>
       </c>
       <c r="BC49" s="5" t="s">
@@ -8683,10 +8683,10 @@
       <c r="BY49" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="BZ49" t="s">
-        <v>6</v>
-      </c>
-      <c r="CA49" t="s">
+      <c r="BZ49" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="CA49" s="25" t="s">
         <v>6</v>
       </c>
       <c r="CB49" s="5" t="s">
@@ -8700,10 +8700,10 @@
       <c r="B50" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C50" t="s">
-        <v>6</v>
-      </c>
-      <c r="D50" t="s">
+      <c r="C50" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="D50" s="25" t="s">
         <v>6</v>
       </c>
       <c r="E50" s="5" t="s">
@@ -8769,10 +8769,10 @@
       <c r="AA50" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="AB50" t="s">
-        <v>6</v>
-      </c>
-      <c r="AC50" t="s">
+      <c r="AB50" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="AC50" s="25" t="s">
         <v>6</v>
       </c>
       <c r="AD50" s="5" t="s">
@@ -8838,10 +8838,10 @@
       <c r="AZ50" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="BA50" t="s">
-        <v>6</v>
-      </c>
-      <c r="BB50" t="s">
+      <c r="BA50" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="BB50" s="25" t="s">
         <v>6</v>
       </c>
       <c r="BC50" s="5" t="s">
@@ -8907,10 +8907,10 @@
       <c r="BY50" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="BZ50" t="s">
-        <v>6</v>
-      </c>
-      <c r="CA50" t="s">
+      <c r="BZ50" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="CA50" s="25" t="s">
         <v>6</v>
       </c>
       <c r="CB50" s="5" t="s">
@@ -8921,10 +8921,10 @@
       <c r="B51" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C51" t="s">
-        <v>6</v>
-      </c>
-      <c r="D51" t="s">
+      <c r="C51" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="D51" s="25" t="s">
         <v>6</v>
       </c>
       <c r="E51" s="5" t="s">
@@ -8963,10 +8963,10 @@
       <c r="AA51" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="AB51" t="s">
-        <v>6</v>
-      </c>
-      <c r="AC51" t="s">
+      <c r="AB51" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="AC51" s="25" t="s">
         <v>6</v>
       </c>
       <c r="AD51" s="5" t="s">
@@ -9005,10 +9005,10 @@
       <c r="AZ51" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="BA51" t="s">
-        <v>6</v>
-      </c>
-      <c r="BB51" t="s">
+      <c r="BA51" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="BB51" s="25" t="s">
         <v>6</v>
       </c>
       <c r="BC51" s="5" t="s">
@@ -9047,10 +9047,10 @@
       <c r="BY51" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="BZ51" t="s">
-        <v>6</v>
-      </c>
-      <c r="CA51" t="s">
+      <c r="BZ51" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="CA51" s="25" t="s">
         <v>6</v>
       </c>
       <c r="CB51" s="5" t="s">
@@ -9225,14 +9225,14 @@
       </c>
     </row>
     <row r="53" spans="1:80" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B53" s="6"/>
-      <c r="C53" s="7"/>
-      <c r="D53" s="22" t="s">
+      <c r="B53" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="E53" s="23" t="s">
+      <c r="C53" s="22" t="s">
         <v>9</v>
       </c>
+      <c r="D53" s="7"/>
+      <c r="E53" s="8"/>
       <c r="F53" t="s">
         <v>8</v>
       </c>
@@ -9272,14 +9272,14 @@
       <c r="Z53" t="s">
         <v>8</v>
       </c>
-      <c r="AA53" s="6"/>
-      <c r="AB53" s="7"/>
-      <c r="AC53" s="22" t="s">
+      <c r="AA53" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="AD53" s="23" t="s">
+      <c r="AB53" s="22" t="s">
         <v>9</v>
       </c>
+      <c r="AC53" s="7"/>
+      <c r="AD53" s="8"/>
       <c r="AE53" t="s">
         <v>8</v>
       </c>
@@ -9319,14 +9319,14 @@
       <c r="AY53" t="s">
         <v>8</v>
       </c>
-      <c r="AZ53" s="6"/>
-      <c r="BA53" s="7"/>
-      <c r="BB53" s="22" t="s">
+      <c r="AZ53" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="BC53" s="23" t="s">
+      <c r="BA53" s="22" t="s">
         <v>9</v>
       </c>
+      <c r="BB53" s="7"/>
+      <c r="BC53" s="8"/>
       <c r="BD53" t="s">
         <v>8</v>
       </c>
@@ -9366,14 +9366,14 @@
       <c r="BX53" t="s">
         <v>8</v>
       </c>
-      <c r="BY53" s="6"/>
-      <c r="BZ53" s="7"/>
-      <c r="CA53" s="22" t="s">
+      <c r="BY53" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="CB53" s="23" t="s">
+      <c r="BZ53" s="22" t="s">
         <v>9</v>
       </c>
+      <c r="CA53" s="7"/>
+      <c r="CB53" s="8"/>
     </row>
     <row r="54" spans="1:80" x14ac:dyDescent="0.35">
       <c r="G54" t="s">
@@ -9738,7 +9738,7 @@
       <c r="W2" s="13"/>
       <c r="X2" s="13"/>
       <c r="Y2" s="14"/>
-      <c r="Z2" s="25"/>
+      <c r="Z2" s="24"/>
       <c r="AA2" s="12" t="s">
         <v>4</v>
       </c>
@@ -15779,7 +15779,7 @@
       <c r="N2" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="O2" s="25"/>
+      <c r="O2" s="24"/>
       <c r="P2" s="12" t="s">
         <v>4</v>
       </c>
@@ -15828,7 +15828,7 @@
       <c r="AM2" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="AN2" s="25"/>
+      <c r="AN2" s="24"/>
       <c r="AO2" s="12" t="s">
         <v>4</v>
       </c>
@@ -15877,7 +15877,7 @@
       <c r="BL2" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="BM2" s="25"/>
+      <c r="BM2" s="24"/>
       <c r="BN2" s="12" t="s">
         <v>4</v>
       </c>
@@ -23641,28 +23641,28 @@
       <c r="BN51" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="BO51" s="26" t="s">
-        <v>0</v>
-      </c>
-      <c r="BP51" s="26" t="s">
-        <v>0</v>
-      </c>
-      <c r="BQ51" s="26" t="s">
-        <v>0</v>
-      </c>
-      <c r="BR51" s="26" t="s">
-        <v>0</v>
-      </c>
-      <c r="BS51" s="26" t="s">
-        <v>0</v>
-      </c>
-      <c r="BT51" s="26" t="s">
-        <v>0</v>
-      </c>
-      <c r="BU51" s="26" t="s">
-        <v>0</v>
-      </c>
-      <c r="BV51" s="26" t="s">
+      <c r="BO51" t="s">
+        <v>0</v>
+      </c>
+      <c r="BP51" t="s">
+        <v>0</v>
+      </c>
+      <c r="BQ51" t="s">
+        <v>0</v>
+      </c>
+      <c r="BR51" t="s">
+        <v>0</v>
+      </c>
+      <c r="BS51" t="s">
+        <v>0</v>
+      </c>
+      <c r="BT51" t="s">
+        <v>0</v>
+      </c>
+      <c r="BU51" t="s">
+        <v>0</v>
+      </c>
+      <c r="BV51" t="s">
         <v>0</v>
       </c>
       <c r="BW51" s="5" t="s">
@@ -23678,13 +23678,6 @@
       </c>
     </row>
     <row r="52" spans="1:81" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B52" s="26"/>
-      <c r="C52" s="26"/>
-      <c r="D52" s="26"/>
-      <c r="E52" s="26"/>
-      <c r="F52" s="26"/>
-      <c r="G52" s="26"/>
-      <c r="H52" s="26"/>
       <c r="I52" s="12" t="s">
         <v>4</v>
       </c>
@@ -23703,25 +23696,8 @@
       <c r="N52" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="O52" s="26"/>
       <c r="P52" s="4"/>
-      <c r="Q52" s="26"/>
-      <c r="R52" s="26"/>
-      <c r="S52" s="26"/>
-      <c r="T52" s="26"/>
-      <c r="U52" s="26"/>
-      <c r="V52" s="26"/>
-      <c r="W52" s="26"/>
-      <c r="X52" s="26"/>
       <c r="Y52" s="5"/>
-      <c r="Z52" s="26"/>
-      <c r="AA52" s="26"/>
-      <c r="AB52" s="26"/>
-      <c r="AC52" s="26"/>
-      <c r="AD52" s="26"/>
-      <c r="AE52" s="26"/>
-      <c r="AF52" s="26"/>
-      <c r="AG52" s="26"/>
       <c r="AH52" s="12" t="s">
         <v>4</v>
       </c>
@@ -23740,25 +23716,8 @@
       <c r="AM52" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="AN52" s="26"/>
       <c r="AO52" s="4"/>
-      <c r="AP52" s="26"/>
-      <c r="AQ52" s="26"/>
-      <c r="AR52" s="26"/>
-      <c r="AS52" s="26"/>
-      <c r="AT52" s="26"/>
-      <c r="AU52" s="26"/>
-      <c r="AV52" s="26"/>
-      <c r="AW52" s="26"/>
       <c r="AX52" s="5"/>
-      <c r="AY52" s="26"/>
-      <c r="AZ52" s="26"/>
-      <c r="BA52" s="26"/>
-      <c r="BB52" s="26"/>
-      <c r="BC52" s="26"/>
-      <c r="BD52" s="26"/>
-      <c r="BE52" s="26"/>
-      <c r="BF52" s="26"/>
       <c r="BG52" s="12" t="s">
         <v>4</v>
       </c>
@@ -23777,7 +23736,6 @@
       <c r="BL52" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="BM52" s="26"/>
       <c r="BN52" s="12"/>
       <c r="BO52" s="13"/>
       <c r="BP52" s="13"/>
@@ -23788,11 +23746,6 @@
       <c r="BU52" s="13"/>
       <c r="BV52" s="13"/>
       <c r="BW52" s="14"/>
-      <c r="BX52" s="26"/>
-      <c r="BY52" s="26"/>
-      <c r="BZ52" s="26"/>
-      <c r="CA52" s="26"/>
-      <c r="CB52" s="26"/>
     </row>
     <row r="53" spans="1:81" x14ac:dyDescent="0.35">
       <c r="O53" s="5" t="s">
@@ -23867,7 +23820,7 @@
       <c r="BL53" t="s">
         <v>7</v>
       </c>
-      <c r="BM53" s="24" t="s">
+      <c r="BM53" s="23" t="s">
         <v>8</v>
       </c>
       <c r="BN53" s="1"/>
@@ -23958,14 +23911,6 @@
         <v>8</v>
       </c>
       <c r="BN54" s="4"/>
-      <c r="BO54" s="26"/>
-      <c r="BP54" s="26"/>
-      <c r="BQ54" s="26"/>
-      <c r="BR54" s="26"/>
-      <c r="BS54" s="26"/>
-      <c r="BT54" s="26"/>
-      <c r="BU54" s="26"/>
-      <c r="BV54" s="26"/>
       <c r="BW54" s="5"/>
     </row>
     <row r="55" spans="1:81" x14ac:dyDescent="0.35">
@@ -24045,14 +23990,6 @@
         <v>8</v>
       </c>
       <c r="BN55" s="4"/>
-      <c r="BO55" s="26"/>
-      <c r="BP55" s="26"/>
-      <c r="BQ55" s="26"/>
-      <c r="BR55" s="26"/>
-      <c r="BS55" s="26"/>
-      <c r="BT55" s="26"/>
-      <c r="BU55" s="26"/>
-      <c r="BV55" s="26"/>
       <c r="BW55" s="5"/>
     </row>
     <row r="56" spans="1:81" x14ac:dyDescent="0.35">
@@ -24132,14 +24069,6 @@
         <v>8</v>
       </c>
       <c r="BN56" s="4"/>
-      <c r="BO56" s="26"/>
-      <c r="BP56" s="26"/>
-      <c r="BQ56" s="26"/>
-      <c r="BR56" s="26"/>
-      <c r="BS56" s="26"/>
-      <c r="BT56" s="26"/>
-      <c r="BU56" s="26"/>
-      <c r="BV56" s="26"/>
       <c r="BW56" s="5"/>
     </row>
     <row r="57" spans="1:81" x14ac:dyDescent="0.35">
@@ -24219,14 +24148,6 @@
         <v>8</v>
       </c>
       <c r="BN57" s="4"/>
-      <c r="BO57" s="26"/>
-      <c r="BP57" s="26"/>
-      <c r="BQ57" s="26"/>
-      <c r="BR57" s="26"/>
-      <c r="BS57" s="26"/>
-      <c r="BT57" s="26"/>
-      <c r="BU57" s="26"/>
-      <c r="BV57" s="26"/>
       <c r="BW57" s="5"/>
     </row>
     <row r="58" spans="1:81" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -24317,7 +24238,6 @@
       <c r="BW58" s="8"/>
     </row>
     <row r="59" spans="1:81" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="O59" s="26"/>
       <c r="P59" s="12" t="s">
         <v>4</v>
       </c>
@@ -24731,7 +24651,7 @@
       <c r="W2" s="13"/>
       <c r="X2" s="13"/>
       <c r="Y2" s="14"/>
-      <c r="Z2" s="25"/>
+      <c r="Z2" s="24"/>
       <c r="AA2" s="12"/>
       <c r="AB2" s="13"/>
       <c r="AC2" s="13"/>
@@ -32472,62 +32392,9 @@
       </c>
     </row>
     <row r="52" spans="1:59" x14ac:dyDescent="0.35">
-      <c r="B52" s="26"/>
-      <c r="C52" s="26"/>
-      <c r="D52" s="26"/>
-      <c r="E52" s="26"/>
-      <c r="F52" s="26"/>
-      <c r="G52" s="26"/>
-      <c r="H52" s="26"/>
-      <c r="I52" s="26"/>
       <c r="J52" s="4"/>
-      <c r="K52" s="26"/>
-      <c r="L52" s="26"/>
-      <c r="M52" s="26"/>
-      <c r="N52" s="26"/>
-      <c r="O52" s="26"/>
-      <c r="P52" s="26"/>
-      <c r="Q52" s="26"/>
-      <c r="R52" s="26"/>
-      <c r="S52" s="26"/>
-      <c r="T52" s="26"/>
-      <c r="U52" s="26"/>
-      <c r="V52" s="26"/>
-      <c r="W52" s="26"/>
-      <c r="X52" s="26"/>
-      <c r="Y52" s="26"/>
       <c r="Z52" s="10"/>
       <c r="AA52" s="4"/>
-      <c r="AB52" s="26"/>
-      <c r="AC52" s="26"/>
-      <c r="AD52" s="26"/>
-      <c r="AE52" s="26"/>
-      <c r="AF52" s="26"/>
-      <c r="AG52" s="26"/>
-      <c r="AH52" s="26"/>
-      <c r="AI52" s="26"/>
-      <c r="AJ52" s="26"/>
-      <c r="AK52" s="26"/>
-      <c r="AL52" s="26"/>
-      <c r="AM52" s="26"/>
-      <c r="AN52" s="26"/>
-      <c r="AO52" s="26"/>
-      <c r="AP52" s="26"/>
-      <c r="AQ52" s="26"/>
-      <c r="AR52" s="26"/>
-      <c r="AS52" s="26"/>
-      <c r="AT52" s="26"/>
-      <c r="AU52" s="26"/>
-      <c r="AV52" s="26"/>
-      <c r="AW52" s="26"/>
-      <c r="AX52" s="26"/>
-      <c r="AY52" s="26"/>
-      <c r="AZ52" s="26"/>
-      <c r="BA52" s="26"/>
-      <c r="BB52" s="26"/>
-      <c r="BC52" s="26"/>
-      <c r="BD52" s="26"/>
-      <c r="BE52" s="26"/>
       <c r="BF52" s="5"/>
     </row>
     <row r="53" spans="1:59" x14ac:dyDescent="0.35">
@@ -33084,7 +32951,7 @@
       <c r="X3" s="13"/>
       <c r="Y3" s="13"/>
       <c r="Z3" s="14"/>
-      <c r="AA3" s="25"/>
+      <c r="AA3" s="24"/>
       <c r="AB3" s="12"/>
       <c r="AC3" s="13"/>
       <c r="AD3" s="13"/>
@@ -33136,7 +33003,7 @@
       <c r="BW3" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="BX3" s="25"/>
+      <c r="BX3" s="24"/>
       <c r="BY3" s="12" t="s">
         <v>4</v>
       </c>
@@ -33185,7 +33052,7 @@
       <c r="CV3" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="CW3" s="25"/>
+      <c r="CW3" s="24"/>
       <c r="CX3" s="12" t="s">
         <v>4</v>
       </c>
@@ -33234,7 +33101,7 @@
       <c r="DU3" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="DV3" s="25"/>
+      <c r="DV3" s="24"/>
       <c r="DW3" s="12" t="s">
         <v>4</v>
       </c>
@@ -48606,28 +48473,28 @@
       <c r="DW52" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="DX52" s="26" t="s">
-        <v>0</v>
-      </c>
-      <c r="DY52" s="26" t="s">
-        <v>0</v>
-      </c>
-      <c r="DZ52" s="26" t="s">
-        <v>0</v>
-      </c>
-      <c r="EA52" s="26" t="s">
-        <v>0</v>
-      </c>
-      <c r="EB52" s="26" t="s">
-        <v>0</v>
-      </c>
-      <c r="EC52" s="26" t="s">
-        <v>0</v>
-      </c>
-      <c r="ED52" s="26" t="s">
-        <v>0</v>
-      </c>
-      <c r="EE52" s="26" t="s">
+      <c r="DX52" t="s">
+        <v>0</v>
+      </c>
+      <c r="DY52" t="s">
+        <v>0</v>
+      </c>
+      <c r="DZ52" t="s">
+        <v>0</v>
+      </c>
+      <c r="EA52" t="s">
+        <v>0</v>
+      </c>
+      <c r="EB52" t="s">
+        <v>0</v>
+      </c>
+      <c r="EC52" t="s">
+        <v>0</v>
+      </c>
+      <c r="ED52" t="s">
+        <v>0</v>
+      </c>
+      <c r="EE52" t="s">
         <v>0</v>
       </c>
       <c r="EF52" s="5" t="s">
@@ -48643,70 +48510,10 @@
       </c>
     </row>
     <row r="53" spans="2:143" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="C53" s="26"/>
-      <c r="D53" s="26"/>
-      <c r="E53" s="26"/>
-      <c r="F53" s="26"/>
-      <c r="G53" s="26"/>
-      <c r="H53" s="26"/>
-      <c r="I53" s="26"/>
-      <c r="J53" s="26"/>
       <c r="K53" s="4"/>
-      <c r="L53" s="26"/>
-      <c r="M53" s="26"/>
-      <c r="N53" s="26"/>
-      <c r="O53" s="26"/>
-      <c r="P53" s="26"/>
-      <c r="Q53" s="26"/>
-      <c r="R53" s="26"/>
-      <c r="S53" s="26"/>
-      <c r="T53" s="26"/>
-      <c r="U53" s="26"/>
-      <c r="V53" s="26"/>
-      <c r="W53" s="26"/>
-      <c r="X53" s="26"/>
-      <c r="Y53" s="26"/>
-      <c r="Z53" s="26"/>
       <c r="AA53" s="10"/>
       <c r="AB53" s="4"/>
-      <c r="AC53" s="26"/>
-      <c r="AD53" s="26"/>
-      <c r="AE53" s="26"/>
-      <c r="AF53" s="26"/>
-      <c r="AG53" s="26"/>
-      <c r="AH53" s="26"/>
-      <c r="AI53" s="26"/>
-      <c r="AJ53" s="26"/>
-      <c r="AK53" s="26"/>
-      <c r="AL53" s="26"/>
-      <c r="AM53" s="26"/>
-      <c r="AN53" s="26"/>
-      <c r="AO53" s="26"/>
-      <c r="AP53" s="26"/>
-      <c r="AQ53" s="26"/>
-      <c r="AR53" s="26"/>
-      <c r="AS53" s="26"/>
-      <c r="AT53" s="26"/>
-      <c r="AU53" s="26"/>
-      <c r="AV53" s="26"/>
-      <c r="AW53" s="26"/>
-      <c r="AX53" s="26"/>
-      <c r="AY53" s="26"/>
-      <c r="AZ53" s="26"/>
-      <c r="BA53" s="26"/>
-      <c r="BB53" s="26"/>
-      <c r="BC53" s="26"/>
-      <c r="BD53" s="26"/>
-      <c r="BE53" s="26"/>
-      <c r="BF53" s="26"/>
       <c r="BG53" s="5"/>
-      <c r="BK53" s="26"/>
-      <c r="BL53" s="26"/>
-      <c r="BM53" s="26"/>
-      <c r="BN53" s="26"/>
-      <c r="BO53" s="26"/>
-      <c r="BP53" s="26"/>
-      <c r="BQ53" s="26"/>
       <c r="BR53" s="12" t="s">
         <v>4</v>
       </c>
@@ -48725,25 +48532,8 @@
       <c r="BW53" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="BX53" s="26"/>
       <c r="BY53" s="4"/>
-      <c r="BZ53" s="26"/>
-      <c r="CA53" s="26"/>
-      <c r="CB53" s="26"/>
-      <c r="CC53" s="26"/>
-      <c r="CD53" s="26"/>
-      <c r="CE53" s="26"/>
-      <c r="CF53" s="26"/>
-      <c r="CG53" s="26"/>
       <c r="CH53" s="5"/>
-      <c r="CI53" s="26"/>
-      <c r="CJ53" s="26"/>
-      <c r="CK53" s="26"/>
-      <c r="CL53" s="26"/>
-      <c r="CM53" s="26"/>
-      <c r="CN53" s="26"/>
-      <c r="CO53" s="26"/>
-      <c r="CP53" s="26"/>
       <c r="CQ53" s="12" t="s">
         <v>4</v>
       </c>
@@ -48762,25 +48552,8 @@
       <c r="CV53" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="CW53" s="26"/>
       <c r="CX53" s="4"/>
-      <c r="CY53" s="26"/>
-      <c r="CZ53" s="26"/>
-      <c r="DA53" s="26"/>
-      <c r="DB53" s="26"/>
-      <c r="DC53" s="26"/>
-      <c r="DD53" s="26"/>
-      <c r="DE53" s="26"/>
-      <c r="DF53" s="26"/>
       <c r="DG53" s="5"/>
-      <c r="DH53" s="26"/>
-      <c r="DI53" s="26"/>
-      <c r="DJ53" s="26"/>
-      <c r="DK53" s="26"/>
-      <c r="DL53" s="26"/>
-      <c r="DM53" s="26"/>
-      <c r="DN53" s="26"/>
-      <c r="DO53" s="26"/>
       <c r="DP53" s="12" t="s">
         <v>4</v>
       </c>
@@ -48799,7 +48572,6 @@
       <c r="DU53" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="DV53" s="26"/>
       <c r="DW53" s="12"/>
       <c r="DX53" s="13"/>
       <c r="DY53" s="13"/>
@@ -48810,11 +48582,6 @@
       <c r="ED53" s="13"/>
       <c r="EE53" s="13"/>
       <c r="EF53" s="14"/>
-      <c r="EG53" s="26"/>
-      <c r="EH53" s="26"/>
-      <c r="EI53" s="26"/>
-      <c r="EJ53" s="26"/>
-      <c r="EK53" s="26"/>
     </row>
     <row r="54" spans="2:143" x14ac:dyDescent="0.35">
       <c r="K54" s="4"/>
@@ -48893,7 +48660,7 @@
       <c r="DU54" t="s">
         <v>7</v>
       </c>
-      <c r="DV54" s="24" t="s">
+      <c r="DV54" s="23" t="s">
         <v>8</v>
       </c>
       <c r="DW54" s="1"/>
@@ -48988,14 +48755,6 @@
         <v>8</v>
       </c>
       <c r="DW55" s="4"/>
-      <c r="DX55" s="26"/>
-      <c r="DY55" s="26"/>
-      <c r="DZ55" s="26"/>
-      <c r="EA55" s="26"/>
-      <c r="EB55" s="26"/>
-      <c r="EC55" s="26"/>
-      <c r="ED55" s="26"/>
-      <c r="EE55" s="26"/>
       <c r="EF55" s="5"/>
     </row>
     <row r="56" spans="2:143" x14ac:dyDescent="0.35">
@@ -49079,14 +48838,6 @@
         <v>8</v>
       </c>
       <c r="DW56" s="4"/>
-      <c r="DX56" s="26"/>
-      <c r="DY56" s="26"/>
-      <c r="DZ56" s="26"/>
-      <c r="EA56" s="26"/>
-      <c r="EB56" s="26"/>
-      <c r="EC56" s="26"/>
-      <c r="ED56" s="26"/>
-      <c r="EE56" s="26"/>
       <c r="EF56" s="5"/>
     </row>
     <row r="57" spans="2:143" x14ac:dyDescent="0.35">
@@ -49170,14 +48921,6 @@
         <v>8</v>
       </c>
       <c r="DW57" s="4"/>
-      <c r="DX57" s="26"/>
-      <c r="DY57" s="26"/>
-      <c r="DZ57" s="26"/>
-      <c r="EA57" s="26"/>
-      <c r="EB57" s="26"/>
-      <c r="EC57" s="26"/>
-      <c r="ED57" s="26"/>
-      <c r="EE57" s="26"/>
       <c r="EF57" s="5"/>
     </row>
     <row r="58" spans="2:143" x14ac:dyDescent="0.35">
@@ -49261,14 +49004,6 @@
         <v>8</v>
       </c>
       <c r="DW58" s="4"/>
-      <c r="DX58" s="26"/>
-      <c r="DY58" s="26"/>
-      <c r="DZ58" s="26"/>
-      <c r="EA58" s="26"/>
-      <c r="EB58" s="26"/>
-      <c r="EC58" s="26"/>
-      <c r="ED58" s="26"/>
-      <c r="EE58" s="26"/>
       <c r="EF58" s="5"/>
     </row>
     <row r="59" spans="2:143" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -49412,7 +49147,6 @@
       <c r="BE60" s="7"/>
       <c r="BF60" s="7"/>
       <c r="BG60" s="8"/>
-      <c r="BX60" s="26"/>
       <c r="BY60" s="12" t="s">
         <v>4</v>
       </c>
@@ -50127,7 +49861,7 @@
       <c r="X64" s="13"/>
       <c r="Y64" s="13"/>
       <c r="Z64" s="14"/>
-      <c r="AA64" s="25"/>
+      <c r="AA64" s="24"/>
       <c r="AB64" s="12" t="s">
         <v>4</v>
       </c>
@@ -51441,10 +51175,10 @@
       <c r="BK69" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="BL69" t="s">
-        <v>6</v>
-      </c>
-      <c r="BM69" t="s">
+      <c r="BL69" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="BM69" s="25" t="s">
         <v>6</v>
       </c>
       <c r="BN69" s="5" t="s">
@@ -51510,10 +51244,10 @@
       <c r="CJ69" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="CK69" t="s">
-        <v>6</v>
-      </c>
-      <c r="CL69" t="s">
+      <c r="CK69" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="CL69" s="25" t="s">
         <v>6</v>
       </c>
       <c r="CM69" s="5" t="s">
@@ -51579,10 +51313,10 @@
       <c r="DI69" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="DJ69" t="s">
-        <v>6</v>
-      </c>
-      <c r="DK69" t="s">
+      <c r="DJ69" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="DK69" s="25" t="s">
         <v>6</v>
       </c>
       <c r="DL69" s="5" t="s">
@@ -51648,10 +51382,10 @@
       <c r="EH69" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="EI69" t="s">
-        <v>6</v>
-      </c>
-      <c r="EJ69" t="s">
+      <c r="EI69" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="EJ69" s="25" t="s">
         <v>6</v>
       </c>
       <c r="EK69" s="5" t="s">
@@ -51836,10 +51570,10 @@
       <c r="BK70" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="BL70" t="s">
-        <v>6</v>
-      </c>
-      <c r="BM70" t="s">
+      <c r="BL70" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="BM70" s="25" t="s">
         <v>6</v>
       </c>
       <c r="BN70" s="5" t="s">
@@ -51905,10 +51639,10 @@
       <c r="CJ70" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="CK70" t="s">
-        <v>6</v>
-      </c>
-      <c r="CL70" t="s">
+      <c r="CK70" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="CL70" s="25" t="s">
         <v>6</v>
       </c>
       <c r="CM70" s="5" t="s">
@@ -51974,10 +51708,10 @@
       <c r="DI70" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="DJ70" t="s">
-        <v>6</v>
-      </c>
-      <c r="DK70" t="s">
+      <c r="DJ70" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="DK70" s="25" t="s">
         <v>6</v>
       </c>
       <c r="DL70" s="5" t="s">
@@ -52043,10 +51777,10 @@
       <c r="EH70" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="EI70" t="s">
-        <v>6</v>
-      </c>
-      <c r="EJ70" t="s">
+      <c r="EI70" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="EJ70" s="25" t="s">
         <v>6</v>
       </c>
       <c r="EK70" s="5" t="s">
@@ -52231,10 +51965,10 @@
       <c r="BK71" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="BL71" t="s">
-        <v>6</v>
-      </c>
-      <c r="BM71" t="s">
+      <c r="BL71" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="BM71" s="25" t="s">
         <v>6</v>
       </c>
       <c r="BN71" s="5" t="s">
@@ -52300,10 +52034,10 @@
       <c r="CJ71" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="CK71" t="s">
-        <v>6</v>
-      </c>
-      <c r="CL71" t="s">
+      <c r="CK71" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="CL71" s="25" t="s">
         <v>6</v>
       </c>
       <c r="CM71" s="5" t="s">
@@ -52369,10 +52103,10 @@
       <c r="DI71" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="DJ71" t="s">
-        <v>6</v>
-      </c>
-      <c r="DK71" t="s">
+      <c r="DJ71" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="DK71" s="25" t="s">
         <v>6</v>
       </c>
       <c r="DL71" s="5" t="s">
@@ -52438,10 +52172,10 @@
       <c r="EH71" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="EI71" t="s">
-        <v>6</v>
-      </c>
-      <c r="EJ71" t="s">
+      <c r="EI71" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="EJ71" s="25" t="s">
         <v>6</v>
       </c>
       <c r="EK71" s="5" t="s">
@@ -52626,10 +52360,10 @@
       <c r="BK72" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="BL72" t="s">
-        <v>6</v>
-      </c>
-      <c r="BM72" t="s">
+      <c r="BL72" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="BM72" s="25" t="s">
         <v>6</v>
       </c>
       <c r="BN72" s="5" t="s">
@@ -52695,10 +52429,10 @@
       <c r="CJ72" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="CK72" t="s">
-        <v>6</v>
-      </c>
-      <c r="CL72" t="s">
+      <c r="CK72" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="CL72" s="25" t="s">
         <v>6</v>
       </c>
       <c r="CM72" s="5" t="s">
@@ -52764,10 +52498,10 @@
       <c r="DI72" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="DJ72" t="s">
-        <v>6</v>
-      </c>
-      <c r="DK72" t="s">
+      <c r="DJ72" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="DK72" s="25" t="s">
         <v>6</v>
       </c>
       <c r="DL72" s="5" t="s">
@@ -52833,10 +52567,10 @@
       <c r="EH72" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="EI72" t="s">
-        <v>6</v>
-      </c>
-      <c r="EJ72" t="s">
+      <c r="EI72" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="EJ72" s="25" t="s">
         <v>6</v>
       </c>
       <c r="EK72" s="5" t="s">
@@ -53022,10 +52756,10 @@
       <c r="BK73" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="BL73" t="s">
-        <v>6</v>
-      </c>
-      <c r="BM73" t="s">
+      <c r="BL73" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="BM73" s="25" t="s">
         <v>6</v>
       </c>
       <c r="BN73" s="5" t="s">
@@ -53091,10 +52825,10 @@
       <c r="CJ73" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="CK73" t="s">
-        <v>6</v>
-      </c>
-      <c r="CL73" t="s">
+      <c r="CK73" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="CL73" s="25" t="s">
         <v>6</v>
       </c>
       <c r="CM73" s="5" t="s">
@@ -53160,10 +52894,10 @@
       <c r="DI73" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="DJ73" t="s">
-        <v>6</v>
-      </c>
-      <c r="DK73" t="s">
+      <c r="DJ73" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="DK73" s="25" t="s">
         <v>6</v>
       </c>
       <c r="DL73" s="5" t="s">
@@ -53229,10 +52963,10 @@
       <c r="EH73" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="EI73" t="s">
-        <v>6</v>
-      </c>
-      <c r="EJ73" t="s">
+      <c r="EI73" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="EJ73" s="25" t="s">
         <v>6</v>
       </c>
       <c r="EK73" s="5" t="s">
@@ -53247,10 +52981,10 @@
       <c r="BK74" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="BL74" t="s">
-        <v>6</v>
-      </c>
-      <c r="BM74" t="s">
+      <c r="BL74" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="BM74" s="25" t="s">
         <v>6</v>
       </c>
       <c r="BN74" s="5" t="s">
@@ -53289,10 +53023,10 @@
       <c r="CJ74" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="CK74" t="s">
-        <v>6</v>
-      </c>
-      <c r="CL74" t="s">
+      <c r="CK74" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="CL74" s="25" t="s">
         <v>6</v>
       </c>
       <c r="CM74" s="5" t="s">
@@ -53331,10 +53065,10 @@
       <c r="DI74" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="DJ74" t="s">
-        <v>6</v>
-      </c>
-      <c r="DK74" t="s">
+      <c r="DJ74" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="DK74" s="25" t="s">
         <v>6</v>
       </c>
       <c r="DL74" s="5" t="s">
@@ -53373,10 +53107,10 @@
       <c r="EH74" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="EI74" t="s">
-        <v>6</v>
-      </c>
-      <c r="EJ74" t="s">
+      <c r="EI74" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="EJ74" s="25" t="s">
         <v>6</v>
       </c>
       <c r="EK74" s="5" t="s">
@@ -53559,14 +53293,14 @@
       <c r="Z76" s="5"/>
       <c r="AB76" s="4"/>
       <c r="BG76" s="5"/>
-      <c r="BK76" s="6"/>
-      <c r="BL76" s="7"/>
-      <c r="BM76" s="22" t="s">
+      <c r="BK76" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="BN76" s="23" t="s">
+      <c r="BL76" s="22" t="s">
         <v>9</v>
       </c>
+      <c r="BM76" s="7"/>
+      <c r="BN76" s="8"/>
       <c r="BO76" t="s">
         <v>8</v>
       </c>
@@ -53606,14 +53340,14 @@
       <c r="CI76" t="s">
         <v>8</v>
       </c>
-      <c r="CJ76" s="6"/>
-      <c r="CK76" s="7"/>
-      <c r="CL76" s="22" t="s">
+      <c r="CJ76" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="CM76" s="23" t="s">
+      <c r="CK76" s="22" t="s">
         <v>9</v>
       </c>
+      <c r="CL76" s="7"/>
+      <c r="CM76" s="8"/>
       <c r="CN76" t="s">
         <v>8</v>
       </c>
@@ -53653,14 +53387,14 @@
       <c r="DH76" t="s">
         <v>8</v>
       </c>
-      <c r="DI76" s="6"/>
-      <c r="DJ76" s="7"/>
-      <c r="DK76" s="22" t="s">
+      <c r="DI76" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="DL76" s="23" t="s">
+      <c r="DJ76" s="22" t="s">
         <v>9</v>
       </c>
+      <c r="DK76" s="7"/>
+      <c r="DL76" s="8"/>
       <c r="DM76" t="s">
         <v>8</v>
       </c>
@@ -53700,14 +53434,14 @@
       <c r="EG76" t="s">
         <v>8</v>
       </c>
-      <c r="EH76" s="6"/>
-      <c r="EI76" s="7"/>
-      <c r="EJ76" s="22" t="s">
+      <c r="EH76" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="EK76" s="23" t="s">
+      <c r="EI76" s="22" t="s">
         <v>9</v>
       </c>
+      <c r="EJ76" s="7"/>
+      <c r="EK76" s="8"/>
       <c r="EM76" s="15"/>
     </row>
     <row r="77" spans="2:143" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -54933,10 +54667,10 @@
       <c r="BK82" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="BL82" t="s">
-        <v>6</v>
-      </c>
-      <c r="BM82" t="s">
+      <c r="BL82" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="BM82" s="25" t="s">
         <v>6</v>
       </c>
       <c r="BN82" s="5" t="s">
@@ -55002,10 +54736,10 @@
       <c r="CJ82" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="CK82" t="s">
-        <v>6</v>
-      </c>
-      <c r="CL82" t="s">
+      <c r="CK82" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="CL82" s="25" t="s">
         <v>6</v>
       </c>
       <c r="CM82" s="5" t="s">
@@ -55071,10 +54805,10 @@
       <c r="DI82" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="DJ82" t="s">
-        <v>6</v>
-      </c>
-      <c r="DK82" t="s">
+      <c r="DJ82" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="DK82" s="25" t="s">
         <v>6</v>
       </c>
       <c r="DL82" s="5" t="s">
@@ -55140,10 +54874,10 @@
       <c r="EH82" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="EI82" t="s">
-        <v>6</v>
-      </c>
-      <c r="EJ82" t="s">
+      <c r="EI82" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="EJ82" s="25" t="s">
         <v>6</v>
       </c>
       <c r="EK82" s="5" t="s">
@@ -55328,10 +55062,10 @@
       <c r="BK83" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="BL83" t="s">
-        <v>6</v>
-      </c>
-      <c r="BM83" t="s">
+      <c r="BL83" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="BM83" s="25" t="s">
         <v>6</v>
       </c>
       <c r="BN83" s="5" t="s">
@@ -55397,10 +55131,10 @@
       <c r="CJ83" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="CK83" t="s">
-        <v>6</v>
-      </c>
-      <c r="CL83" t="s">
+      <c r="CK83" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="CL83" s="25" t="s">
         <v>6</v>
       </c>
       <c r="CM83" s="5" t="s">
@@ -55466,10 +55200,10 @@
       <c r="DI83" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="DJ83" t="s">
-        <v>6</v>
-      </c>
-      <c r="DK83" t="s">
+      <c r="DJ83" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="DK83" s="25" t="s">
         <v>6</v>
       </c>
       <c r="DL83" s="5" t="s">
@@ -55535,10 +55269,10 @@
       <c r="EH83" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="EI83" t="s">
-        <v>6</v>
-      </c>
-      <c r="EJ83" t="s">
+      <c r="EI83" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="EJ83" s="25" t="s">
         <v>6</v>
       </c>
       <c r="EK83" s="5" t="s">
@@ -55723,10 +55457,10 @@
       <c r="BK84" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="BL84" t="s">
-        <v>6</v>
-      </c>
-      <c r="BM84" t="s">
+      <c r="BL84" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="BM84" s="25" t="s">
         <v>6</v>
       </c>
       <c r="BN84" s="5" t="s">
@@ -55792,10 +55526,10 @@
       <c r="CJ84" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="CK84" t="s">
-        <v>6</v>
-      </c>
-      <c r="CL84" t="s">
+      <c r="CK84" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="CL84" s="25" t="s">
         <v>6</v>
       </c>
       <c r="CM84" s="5" t="s">
@@ -55861,10 +55595,10 @@
       <c r="DI84" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="DJ84" t="s">
-        <v>6</v>
-      </c>
-      <c r="DK84" t="s">
+      <c r="DJ84" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="DK84" s="25" t="s">
         <v>6</v>
       </c>
       <c r="DL84" s="5" t="s">
@@ -55930,10 +55664,10 @@
       <c r="EH84" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="EI84" t="s">
-        <v>6</v>
-      </c>
-      <c r="EJ84" t="s">
+      <c r="EI84" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="EJ84" s="25" t="s">
         <v>6</v>
       </c>
       <c r="EK84" s="5" t="s">
@@ -56118,10 +55852,10 @@
       <c r="BK85" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="BL85" t="s">
-        <v>6</v>
-      </c>
-      <c r="BM85" t="s">
+      <c r="BL85" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="BM85" s="25" t="s">
         <v>6</v>
       </c>
       <c r="BN85" s="5" t="s">
@@ -56187,10 +55921,10 @@
       <c r="CJ85" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="CK85" t="s">
-        <v>6</v>
-      </c>
-      <c r="CL85" t="s">
+      <c r="CK85" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="CL85" s="25" t="s">
         <v>6</v>
       </c>
       <c r="CM85" s="5" t="s">
@@ -56256,10 +55990,10 @@
       <c r="DI85" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="DJ85" t="s">
-        <v>6</v>
-      </c>
-      <c r="DK85" t="s">
+      <c r="DJ85" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="DK85" s="25" t="s">
         <v>6</v>
       </c>
       <c r="DL85" s="5" t="s">
@@ -56325,10 +56059,10 @@
       <c r="EH85" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="EI85" t="s">
-        <v>6</v>
-      </c>
-      <c r="EJ85" t="s">
+      <c r="EI85" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="EJ85" s="25" t="s">
         <v>6</v>
       </c>
       <c r="EK85" s="5" t="s">
@@ -56514,10 +56248,10 @@
       <c r="BK86" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="BL86" t="s">
-        <v>6</v>
-      </c>
-      <c r="BM86" t="s">
+      <c r="BL86" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="BM86" s="25" t="s">
         <v>6</v>
       </c>
       <c r="BN86" s="5" t="s">
@@ -56583,10 +56317,10 @@
       <c r="CJ86" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="CK86" t="s">
-        <v>6</v>
-      </c>
-      <c r="CL86" t="s">
+      <c r="CK86" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="CL86" s="25" t="s">
         <v>6</v>
       </c>
       <c r="CM86" s="5" t="s">
@@ -56652,10 +56386,10 @@
       <c r="DI86" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="DJ86" t="s">
-        <v>6</v>
-      </c>
-      <c r="DK86" t="s">
+      <c r="DJ86" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="DK86" s="25" t="s">
         <v>6</v>
       </c>
       <c r="DL86" s="5" t="s">
@@ -56721,10 +56455,10 @@
       <c r="EH86" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="EI86" t="s">
-        <v>6</v>
-      </c>
-      <c r="EJ86" t="s">
+      <c r="EI86" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="EJ86" s="25" t="s">
         <v>6</v>
       </c>
       <c r="EK86" s="5" t="s">
@@ -56739,10 +56473,10 @@
       <c r="BK87" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="BL87" t="s">
-        <v>6</v>
-      </c>
-      <c r="BM87" t="s">
+      <c r="BL87" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="BM87" s="25" t="s">
         <v>6</v>
       </c>
       <c r="BN87" s="5" t="s">
@@ -56781,10 +56515,10 @@
       <c r="CJ87" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="CK87" t="s">
-        <v>6</v>
-      </c>
-      <c r="CL87" t="s">
+      <c r="CK87" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="CL87" s="25" t="s">
         <v>6</v>
       </c>
       <c r="CM87" s="5" t="s">
@@ -56823,10 +56557,10 @@
       <c r="DI87" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="DJ87" t="s">
-        <v>6</v>
-      </c>
-      <c r="DK87" t="s">
+      <c r="DJ87" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="DK87" s="25" t="s">
         <v>6</v>
       </c>
       <c r="DL87" s="5" t="s">
@@ -56865,10 +56599,10 @@
       <c r="EH87" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="EI87" t="s">
-        <v>6</v>
-      </c>
-      <c r="EJ87" t="s">
+      <c r="EI87" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="EJ87" s="25" t="s">
         <v>6</v>
       </c>
       <c r="EK87" s="5" t="s">
@@ -57051,14 +56785,14 @@
       <c r="Z89" s="5"/>
       <c r="AB89" s="4"/>
       <c r="BG89" s="5"/>
-      <c r="BK89" s="6"/>
-      <c r="BL89" s="7"/>
-      <c r="BM89" s="22" t="s">
+      <c r="BK89" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="BN89" s="23" t="s">
+      <c r="BL89" s="22" t="s">
         <v>9</v>
       </c>
+      <c r="BM89" s="7"/>
+      <c r="BN89" s="8"/>
       <c r="BO89" t="s">
         <v>8</v>
       </c>
@@ -57098,14 +56832,14 @@
       <c r="CI89" t="s">
         <v>8</v>
       </c>
-      <c r="CJ89" s="6"/>
-      <c r="CK89" s="7"/>
-      <c r="CL89" s="22" t="s">
+      <c r="CJ89" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="CM89" s="23" t="s">
+      <c r="CK89" s="22" t="s">
         <v>9</v>
       </c>
+      <c r="CL89" s="7"/>
+      <c r="CM89" s="8"/>
       <c r="CN89" t="s">
         <v>8</v>
       </c>
@@ -57145,14 +56879,14 @@
       <c r="DH89" t="s">
         <v>8</v>
       </c>
-      <c r="DI89" s="6"/>
-      <c r="DJ89" s="7"/>
-      <c r="DK89" s="22" t="s">
+      <c r="DI89" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="DL89" s="23" t="s">
+      <c r="DJ89" s="22" t="s">
         <v>9</v>
       </c>
+      <c r="DK89" s="7"/>
+      <c r="DL89" s="8"/>
       <c r="DM89" t="s">
         <v>8</v>
       </c>
@@ -57192,14 +56926,14 @@
       <c r="EG89" t="s">
         <v>8</v>
       </c>
-      <c r="EH89" s="6"/>
-      <c r="EI89" s="7"/>
-      <c r="EJ89" s="22" t="s">
+      <c r="EH89" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="EK89" s="23" t="s">
+      <c r="EI89" s="22" t="s">
         <v>9</v>
       </c>
+      <c r="EJ89" s="7"/>
+      <c r="EK89" s="8"/>
       <c r="EM89" s="15"/>
     </row>
     <row r="90" spans="2:143" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -58425,10 +58159,10 @@
       <c r="BK95" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="BL95" t="s">
-        <v>6</v>
-      </c>
-      <c r="BM95" t="s">
+      <c r="BL95" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="BM95" s="25" t="s">
         <v>6</v>
       </c>
       <c r="BN95" s="5" t="s">
@@ -58494,10 +58228,10 @@
       <c r="CJ95" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="CK95" t="s">
-        <v>6</v>
-      </c>
-      <c r="CL95" t="s">
+      <c r="CK95" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="CL95" s="25" t="s">
         <v>6</v>
       </c>
       <c r="CM95" s="5" t="s">
@@ -58563,10 +58297,10 @@
       <c r="DI95" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="DJ95" t="s">
-        <v>6</v>
-      </c>
-      <c r="DK95" t="s">
+      <c r="DJ95" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="DK95" s="25" t="s">
         <v>6</v>
       </c>
       <c r="DL95" s="5" t="s">
@@ -58632,10 +58366,10 @@
       <c r="EH95" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="EI95" t="s">
-        <v>6</v>
-      </c>
-      <c r="EJ95" t="s">
+      <c r="EI95" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="EJ95" s="25" t="s">
         <v>6</v>
       </c>
       <c r="EK95" s="5" t="s">
@@ -58820,10 +58554,10 @@
       <c r="BK96" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="BL96" t="s">
-        <v>6</v>
-      </c>
-      <c r="BM96" t="s">
+      <c r="BL96" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="BM96" s="25" t="s">
         <v>6</v>
       </c>
       <c r="BN96" s="5" t="s">
@@ -58889,10 +58623,10 @@
       <c r="CJ96" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="CK96" t="s">
-        <v>6</v>
-      </c>
-      <c r="CL96" t="s">
+      <c r="CK96" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="CL96" s="25" t="s">
         <v>6</v>
       </c>
       <c r="CM96" s="5" t="s">
@@ -58958,10 +58692,10 @@
       <c r="DI96" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="DJ96" t="s">
-        <v>6</v>
-      </c>
-      <c r="DK96" t="s">
+      <c r="DJ96" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="DK96" s="25" t="s">
         <v>6</v>
       </c>
       <c r="DL96" s="5" t="s">
@@ -59027,10 +58761,10 @@
       <c r="EH96" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="EI96" t="s">
-        <v>6</v>
-      </c>
-      <c r="EJ96" t="s">
+      <c r="EI96" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="EJ96" s="25" t="s">
         <v>6</v>
       </c>
       <c r="EK96" s="5" t="s">
@@ -59215,10 +58949,10 @@
       <c r="BK97" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="BL97" t="s">
-        <v>6</v>
-      </c>
-      <c r="BM97" t="s">
+      <c r="BL97" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="BM97" s="25" t="s">
         <v>6</v>
       </c>
       <c r="BN97" s="5" t="s">
@@ -59284,10 +59018,10 @@
       <c r="CJ97" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="CK97" t="s">
-        <v>6</v>
-      </c>
-      <c r="CL97" t="s">
+      <c r="CK97" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="CL97" s="25" t="s">
         <v>6</v>
       </c>
       <c r="CM97" s="5" t="s">
@@ -59353,10 +59087,10 @@
       <c r="DI97" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="DJ97" t="s">
-        <v>6</v>
-      </c>
-      <c r="DK97" t="s">
+      <c r="DJ97" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="DK97" s="25" t="s">
         <v>6</v>
       </c>
       <c r="DL97" s="5" t="s">
@@ -59422,10 +59156,10 @@
       <c r="EH97" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="EI97" t="s">
-        <v>6</v>
-      </c>
-      <c r="EJ97" t="s">
+      <c r="EI97" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="EJ97" s="25" t="s">
         <v>6</v>
       </c>
       <c r="EK97" s="5" t="s">
@@ -59610,10 +59344,10 @@
       <c r="BK98" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="BL98" t="s">
-        <v>6</v>
-      </c>
-      <c r="BM98" t="s">
+      <c r="BL98" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="BM98" s="25" t="s">
         <v>6</v>
       </c>
       <c r="BN98" s="5" t="s">
@@ -59679,10 +59413,10 @@
       <c r="CJ98" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="CK98" t="s">
-        <v>6</v>
-      </c>
-      <c r="CL98" t="s">
+      <c r="CK98" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="CL98" s="25" t="s">
         <v>6</v>
       </c>
       <c r="CM98" s="5" t="s">
@@ -59748,10 +59482,10 @@
       <c r="DI98" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="DJ98" t="s">
-        <v>6</v>
-      </c>
-      <c r="DK98" t="s">
+      <c r="DJ98" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="DK98" s="25" t="s">
         <v>6</v>
       </c>
       <c r="DL98" s="5" t="s">
@@ -59817,10 +59551,10 @@
       <c r="EH98" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="EI98" t="s">
-        <v>6</v>
-      </c>
-      <c r="EJ98" t="s">
+      <c r="EI98" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="EJ98" s="25" t="s">
         <v>6</v>
       </c>
       <c r="EK98" s="5" t="s">
@@ -60006,10 +59740,10 @@
       <c r="BK99" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="BL99" t="s">
-        <v>6</v>
-      </c>
-      <c r="BM99" t="s">
+      <c r="BL99" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="BM99" s="25" t="s">
         <v>6</v>
       </c>
       <c r="BN99" s="5" t="s">
@@ -60075,10 +59809,10 @@
       <c r="CJ99" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="CK99" t="s">
-        <v>6</v>
-      </c>
-      <c r="CL99" t="s">
+      <c r="CK99" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="CL99" s="25" t="s">
         <v>6</v>
       </c>
       <c r="CM99" s="5" t="s">
@@ -60144,10 +59878,10 @@
       <c r="DI99" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="DJ99" t="s">
-        <v>6</v>
-      </c>
-      <c r="DK99" t="s">
+      <c r="DJ99" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="DK99" s="25" t="s">
         <v>6</v>
       </c>
       <c r="DL99" s="5" t="s">
@@ -60213,10 +59947,10 @@
       <c r="EH99" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="EI99" t="s">
-        <v>6</v>
-      </c>
-      <c r="EJ99" t="s">
+      <c r="EI99" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="EJ99" s="25" t="s">
         <v>6</v>
       </c>
       <c r="EK99" s="5" t="s">
@@ -60231,10 +59965,10 @@
       <c r="BK100" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="BL100" t="s">
-        <v>6</v>
-      </c>
-      <c r="BM100" t="s">
+      <c r="BL100" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="BM100" s="25" t="s">
         <v>6</v>
       </c>
       <c r="BN100" s="5" t="s">
@@ -60273,10 +60007,10 @@
       <c r="CJ100" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="CK100" t="s">
-        <v>6</v>
-      </c>
-      <c r="CL100" t="s">
+      <c r="CK100" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="CL100" s="25" t="s">
         <v>6</v>
       </c>
       <c r="CM100" s="5" t="s">
@@ -60315,10 +60049,10 @@
       <c r="DI100" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="DJ100" t="s">
-        <v>6</v>
-      </c>
-      <c r="DK100" t="s">
+      <c r="DJ100" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="DK100" s="25" t="s">
         <v>6</v>
       </c>
       <c r="DL100" s="5" t="s">
@@ -60357,10 +60091,10 @@
       <c r="EH100" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="EI100" t="s">
-        <v>6</v>
-      </c>
-      <c r="EJ100" t="s">
+      <c r="EI100" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="EJ100" s="25" t="s">
         <v>6</v>
       </c>
       <c r="EK100" s="5" t="s">
@@ -60543,14 +60277,14 @@
       <c r="Z102" s="5"/>
       <c r="AB102" s="4"/>
       <c r="BG102" s="5"/>
-      <c r="BK102" s="6"/>
-      <c r="BL102" s="7"/>
-      <c r="BM102" s="22" t="s">
+      <c r="BK102" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="BN102" s="23" t="s">
+      <c r="BL102" s="22" t="s">
         <v>9</v>
       </c>
+      <c r="BM102" s="7"/>
+      <c r="BN102" s="8"/>
       <c r="BO102" t="s">
         <v>8</v>
       </c>
@@ -60590,14 +60324,14 @@
       <c r="CI102" t="s">
         <v>8</v>
       </c>
-      <c r="CJ102" s="6"/>
-      <c r="CK102" s="7"/>
-      <c r="CL102" s="22" t="s">
+      <c r="CJ102" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="CM102" s="23" t="s">
+      <c r="CK102" s="22" t="s">
         <v>9</v>
       </c>
+      <c r="CL102" s="7"/>
+      <c r="CM102" s="8"/>
       <c r="CN102" t="s">
         <v>8</v>
       </c>
@@ -60637,14 +60371,14 @@
       <c r="DH102" t="s">
         <v>8</v>
       </c>
-      <c r="DI102" s="6"/>
-      <c r="DJ102" s="7"/>
-      <c r="DK102" s="22" t="s">
+      <c r="DI102" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="DL102" s="23" t="s">
+      <c r="DJ102" s="22" t="s">
         <v>9</v>
       </c>
+      <c r="DK102" s="7"/>
+      <c r="DL102" s="8"/>
       <c r="DM102" t="s">
         <v>8</v>
       </c>
@@ -60684,14 +60418,14 @@
       <c r="EG102" t="s">
         <v>8</v>
       </c>
-      <c r="EH102" s="6"/>
-      <c r="EI102" s="7"/>
-      <c r="EJ102" s="22" t="s">
+      <c r="EH102" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="EK102" s="23" t="s">
+      <c r="EI102" s="22" t="s">
         <v>9</v>
       </c>
+      <c r="EJ102" s="7"/>
+      <c r="EK102" s="8"/>
       <c r="EM102" s="15"/>
     </row>
     <row r="103" spans="2:143" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -61917,10 +61651,10 @@
       <c r="BK108" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="BL108" t="s">
-        <v>6</v>
-      </c>
-      <c r="BM108" t="s">
+      <c r="BL108" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="BM108" s="25" t="s">
         <v>6</v>
       </c>
       <c r="BN108" s="5" t="s">
@@ -61986,10 +61720,10 @@
       <c r="CJ108" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="CK108" t="s">
-        <v>6</v>
-      </c>
-      <c r="CL108" t="s">
+      <c r="CK108" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="CL108" s="25" t="s">
         <v>6</v>
       </c>
       <c r="CM108" s="5" t="s">
@@ -62055,10 +61789,10 @@
       <c r="DI108" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="DJ108" t="s">
-        <v>6</v>
-      </c>
-      <c r="DK108" t="s">
+      <c r="DJ108" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="DK108" s="25" t="s">
         <v>6</v>
       </c>
       <c r="DL108" s="5" t="s">
@@ -62124,10 +61858,10 @@
       <c r="EH108" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="EI108" t="s">
-        <v>6</v>
-      </c>
-      <c r="EJ108" t="s">
+      <c r="EI108" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="EJ108" s="25" t="s">
         <v>6</v>
       </c>
       <c r="EK108" s="5" t="s">
@@ -62312,10 +62046,10 @@
       <c r="BK109" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="BL109" t="s">
-        <v>6</v>
-      </c>
-      <c r="BM109" t="s">
+      <c r="BL109" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="BM109" s="25" t="s">
         <v>6</v>
       </c>
       <c r="BN109" s="5" t="s">
@@ -62381,10 +62115,10 @@
       <c r="CJ109" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="CK109" t="s">
-        <v>6</v>
-      </c>
-      <c r="CL109" t="s">
+      <c r="CK109" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="CL109" s="25" t="s">
         <v>6</v>
       </c>
       <c r="CM109" s="5" t="s">
@@ -62450,10 +62184,10 @@
       <c r="DI109" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="DJ109" t="s">
-        <v>6</v>
-      </c>
-      <c r="DK109" t="s">
+      <c r="DJ109" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="DK109" s="25" t="s">
         <v>6</v>
       </c>
       <c r="DL109" s="5" t="s">
@@ -62519,10 +62253,10 @@
       <c r="EH109" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="EI109" t="s">
-        <v>6</v>
-      </c>
-      <c r="EJ109" t="s">
+      <c r="EI109" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="EJ109" s="25" t="s">
         <v>6</v>
       </c>
       <c r="EK109" s="5" t="s">
@@ -62707,10 +62441,10 @@
       <c r="BK110" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="BL110" t="s">
-        <v>6</v>
-      </c>
-      <c r="BM110" t="s">
+      <c r="BL110" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="BM110" s="25" t="s">
         <v>6</v>
       </c>
       <c r="BN110" s="5" t="s">
@@ -62776,10 +62510,10 @@
       <c r="CJ110" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="CK110" t="s">
-        <v>6</v>
-      </c>
-      <c r="CL110" t="s">
+      <c r="CK110" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="CL110" s="25" t="s">
         <v>6</v>
       </c>
       <c r="CM110" s="5" t="s">
@@ -62845,10 +62579,10 @@
       <c r="DI110" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="DJ110" t="s">
-        <v>6</v>
-      </c>
-      <c r="DK110" t="s">
+      <c r="DJ110" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="DK110" s="25" t="s">
         <v>6</v>
       </c>
       <c r="DL110" s="5" t="s">
@@ -62914,10 +62648,10 @@
       <c r="EH110" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="EI110" t="s">
-        <v>6</v>
-      </c>
-      <c r="EJ110" t="s">
+      <c r="EI110" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="EJ110" s="25" t="s">
         <v>6</v>
       </c>
       <c r="EK110" s="5" t="s">
@@ -63102,10 +62836,10 @@
       <c r="BK111" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="BL111" t="s">
-        <v>6</v>
-      </c>
-      <c r="BM111" t="s">
+      <c r="BL111" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="BM111" s="25" t="s">
         <v>6</v>
       </c>
       <c r="BN111" s="5" t="s">
@@ -63171,10 +62905,10 @@
       <c r="CJ111" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="CK111" t="s">
-        <v>6</v>
-      </c>
-      <c r="CL111" t="s">
+      <c r="CK111" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="CL111" s="25" t="s">
         <v>6</v>
       </c>
       <c r="CM111" s="5" t="s">
@@ -63240,10 +62974,10 @@
       <c r="DI111" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="DJ111" t="s">
-        <v>6</v>
-      </c>
-      <c r="DK111" t="s">
+      <c r="DJ111" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="DK111" s="25" t="s">
         <v>6</v>
       </c>
       <c r="DL111" s="5" t="s">
@@ -63309,10 +63043,10 @@
       <c r="EH111" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="EI111" t="s">
-        <v>6</v>
-      </c>
-      <c r="EJ111" t="s">
+      <c r="EI111" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="EJ111" s="25" t="s">
         <v>6</v>
       </c>
       <c r="EK111" s="5" t="s">
@@ -63497,10 +63231,10 @@
       <c r="BK112" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="BL112" t="s">
-        <v>6</v>
-      </c>
-      <c r="BM112" t="s">
+      <c r="BL112" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="BM112" s="25" t="s">
         <v>6</v>
       </c>
       <c r="BN112" s="5" t="s">
@@ -63566,10 +63300,10 @@
       <c r="CJ112" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="CK112" t="s">
-        <v>6</v>
-      </c>
-      <c r="CL112" t="s">
+      <c r="CK112" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="CL112" s="25" t="s">
         <v>6</v>
       </c>
       <c r="CM112" s="5" t="s">
@@ -63635,10 +63369,10 @@
       <c r="DI112" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="DJ112" t="s">
-        <v>6</v>
-      </c>
-      <c r="DK112" t="s">
+      <c r="DJ112" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="DK112" s="25" t="s">
         <v>6</v>
       </c>
       <c r="DL112" s="5" t="s">
@@ -63704,10 +63438,10 @@
       <c r="EH112" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="EI112" t="s">
-        <v>6</v>
-      </c>
-      <c r="EJ112" t="s">
+      <c r="EI112" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="EJ112" s="25" t="s">
         <v>6</v>
       </c>
       <c r="EK112" s="5" t="s">
@@ -63745,10 +63479,10 @@
       <c r="BK113" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="BL113" t="s">
-        <v>6</v>
-      </c>
-      <c r="BM113" t="s">
+      <c r="BL113" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="BM113" s="25" t="s">
         <v>6</v>
       </c>
       <c r="BN113" s="5" t="s">
@@ -63787,10 +63521,10 @@
       <c r="CJ113" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="CK113" t="s">
-        <v>6</v>
-      </c>
-      <c r="CL113" t="s">
+      <c r="CK113" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="CL113" s="25" t="s">
         <v>6</v>
       </c>
       <c r="CM113" s="5" t="s">
@@ -63829,10 +63563,10 @@
       <c r="DI113" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="DJ113" t="s">
-        <v>6</v>
-      </c>
-      <c r="DK113" t="s">
+      <c r="DJ113" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="DK113" s="25" t="s">
         <v>6</v>
       </c>
       <c r="DL113" s="5" t="s">
@@ -63871,10 +63605,10 @@
       <c r="EH113" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="EI113" t="s">
-        <v>6</v>
-      </c>
-      <c r="EJ113" t="s">
+      <c r="EI113" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="EJ113" s="25" t="s">
         <v>6</v>
       </c>
       <c r="EK113" s="5" t="s">
@@ -64133,14 +63867,14 @@
       <c r="BE115" s="7"/>
       <c r="BF115" s="7"/>
       <c r="BG115" s="8"/>
-      <c r="BK115" s="6"/>
-      <c r="BL115" s="7"/>
-      <c r="BM115" s="22" t="s">
+      <c r="BK115" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="BN115" s="23" t="s">
+      <c r="BL115" s="22" t="s">
         <v>9</v>
       </c>
+      <c r="BM115" s="7"/>
+      <c r="BN115" s="8"/>
       <c r="BO115" t="s">
         <v>8</v>
       </c>
@@ -64180,14 +63914,14 @@
       <c r="CI115" t="s">
         <v>8</v>
       </c>
-      <c r="CJ115" s="6"/>
-      <c r="CK115" s="7"/>
-      <c r="CL115" s="22" t="s">
+      <c r="CJ115" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="CM115" s="23" t="s">
+      <c r="CK115" s="22" t="s">
         <v>9</v>
       </c>
+      <c r="CL115" s="7"/>
+      <c r="CM115" s="8"/>
       <c r="CN115" t="s">
         <v>8</v>
       </c>
@@ -64227,14 +63961,14 @@
       <c r="DH115" t="s">
         <v>8</v>
       </c>
-      <c r="DI115" s="6"/>
-      <c r="DJ115" s="7"/>
-      <c r="DK115" s="22" t="s">
+      <c r="DI115" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="DL115" s="23" t="s">
+      <c r="DJ115" s="22" t="s">
         <v>9</v>
       </c>
+      <c r="DK115" s="7"/>
+      <c r="DL115" s="8"/>
       <c r="DM115" t="s">
         <v>8</v>
       </c>
@@ -64274,14 +64008,14 @@
       <c r="EG115" t="s">
         <v>8</v>
       </c>
-      <c r="EH115" s="6"/>
-      <c r="EI115" s="7"/>
-      <c r="EJ115" s="22" t="s">
+      <c r="EH115" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="EK115" s="23" t="s">
+      <c r="EI115" s="22" t="s">
         <v>9</v>
       </c>
+      <c r="EJ115" s="7"/>
+      <c r="EK115" s="8"/>
     </row>
     <row r="116" spans="3:141" x14ac:dyDescent="0.35">
       <c r="K116" t="s">

</xml_diff>

<commit_message>
Fixed more routing mess
</commit_message>
<xml_diff>
--- a/Configuration Generator/Layout Drawings.xlsx
+++ b/Configuration Generator/Layout Drawings.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/13561f3231cadc0a/DTU/Comp_Arch_2/eFPGA/Configuration Generator/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="871" documentId="13_ncr:1_{FB05B031-63D2-4F22-8938-A1D344FEFB29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{241B9AB7-2059-41BE-A42A-D90D18FB78EB}"/>
+  <xr:revisionPtr revIDLastSave="889" documentId="13_ncr:1_{FB05B031-63D2-4F22-8938-A1D344FEFB29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{FFF21129-7776-4824-B8D2-FD9DA643D7B9}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23891,7 +23891,7 @@
       <c r="Y53" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="AM53" t="s">
+      <c r="AH53" t="s">
         <v>6</v>
       </c>
       <c r="AN53" s="5" t="s">
@@ -23927,7 +23927,7 @@
       <c r="AX53" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="BL53" t="s">
+      <c r="BG53" t="s">
         <v>6</v>
       </c>
       <c r="BM53" s="23" t="s">
@@ -23978,7 +23978,7 @@
       <c r="Y54" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="AL54" t="s">
+      <c r="AI54" t="s">
         <v>6</v>
       </c>
       <c r="AN54" s="5" t="s">
@@ -24014,7 +24014,7 @@
       <c r="AX54" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="BK54" t="s">
+      <c r="BH54" t="s">
         <v>6</v>
       </c>
       <c r="BM54" t="s">
@@ -24057,7 +24057,7 @@
       <c r="Y55" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="AK55" t="s">
+      <c r="AJ55" t="s">
         <v>6</v>
       </c>
       <c r="AN55" t="s">
@@ -24093,7 +24093,7 @@
       <c r="AX55" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="BJ55" t="s">
+      <c r="BI55" t="s">
         <v>6</v>
       </c>
       <c r="BM55" t="s">
@@ -24136,7 +24136,7 @@
       <c r="Y56" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="AJ56" t="s">
+      <c r="AK56" t="s">
         <v>6</v>
       </c>
       <c r="AN56" t="s">
@@ -24172,7 +24172,7 @@
       <c r="AX56" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="BI56" t="s">
+      <c r="BJ56" t="s">
         <v>6</v>
       </c>
       <c r="BM56" t="s">
@@ -24215,7 +24215,7 @@
       <c r="Y57" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="AI57" t="s">
+      <c r="AL57" t="s">
         <v>6</v>
       </c>
       <c r="AN57" t="s">
@@ -24251,7 +24251,7 @@
       <c r="AX57" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="BH57" t="s">
+      <c r="BK57" t="s">
         <v>6</v>
       </c>
       <c r="BM57" t="s">
@@ -24294,7 +24294,7 @@
       <c r="Y58" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="AH58" t="s">
+      <c r="AM58" t="s">
         <v>6</v>
       </c>
       <c r="AN58" t="s">
@@ -24330,7 +24330,7 @@
       <c r="AX58" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="BG58" t="s">
+      <c r="BL58" t="s">
         <v>6</v>
       </c>
       <c r="BM58" t="s">
@@ -48737,7 +48737,7 @@
       <c r="CH54" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="CV54" t="s">
+      <c r="CQ54" t="s">
         <v>6</v>
       </c>
       <c r="CW54" s="5" t="s">
@@ -48773,7 +48773,7 @@
       <c r="DG54" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="DU54" t="s">
+      <c r="DP54" t="s">
         <v>6</v>
       </c>
       <c r="DV54" s="23" t="s">
@@ -48828,7 +48828,7 @@
       <c r="CH55" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="CU55" t="s">
+      <c r="CR55" t="s">
         <v>6</v>
       </c>
       <c r="CW55" s="5" t="s">
@@ -48864,7 +48864,7 @@
       <c r="DG55" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="DT55" t="s">
+      <c r="DQ55" t="s">
         <v>6</v>
       </c>
       <c r="DV55" t="s">
@@ -48911,7 +48911,7 @@
       <c r="CH56" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="CT56" t="s">
+      <c r="CS56" t="s">
         <v>6</v>
       </c>
       <c r="CW56" t="s">
@@ -48947,7 +48947,7 @@
       <c r="DG56" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="DS56" t="s">
+      <c r="DR56" t="s">
         <v>6</v>
       </c>
       <c r="DV56" t="s">
@@ -48994,7 +48994,7 @@
       <c r="CH57" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="CS57" t="s">
+      <c r="CT57" t="s">
         <v>6</v>
       </c>
       <c r="CW57" t="s">
@@ -49030,7 +49030,7 @@
       <c r="DG57" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="DR57" t="s">
+      <c r="DS57" t="s">
         <v>6</v>
       </c>
       <c r="DV57" t="s">
@@ -49077,7 +49077,7 @@
       <c r="CH58" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="CR58" t="s">
+      <c r="CU58" t="s">
         <v>6</v>
       </c>
       <c r="CW58" t="s">
@@ -49113,7 +49113,7 @@
       <c r="DG58" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="DQ58" t="s">
+      <c r="DT58" t="s">
         <v>6</v>
       </c>
       <c r="DV58" t="s">
@@ -49160,7 +49160,7 @@
       <c r="CH59" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="CQ59" t="s">
+      <c r="CV59" t="s">
         <v>6</v>
       </c>
       <c r="CW59" t="s">
@@ -49196,7 +49196,7 @@
       <c r="DG59" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="DP59" t="s">
+      <c r="DU59" t="s">
         <v>6</v>
       </c>
       <c r="DV59" t="s">

</xml_diff>